<commit_message>
build: regenerate spreadsheet with partial Europe enrichment
</commit_message>
<xml_diff>
--- a/watch-microbrand-database.xlsx
+++ b/watch-microbrand-database.xlsx
@@ -469,35 +469,35 @@
       <c r="C2" t="str">
         <v>Paris</v>
       </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-      <c r="F2" t="str">
-        <v/>
+      <c r="D2">
+        <v>2024</v>
+      </c>
+      <c r="E2">
+        <v>1703</v>
+      </c>
+      <c r="F2">
+        <v>1919</v>
       </c>
       <c r="G2" t="str">
         <v>Active</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>2026 Millésime (Edmond &amp; Arsène)</v>
       </c>
       <c r="I2" t="str">
-        <v/>
+        <v>2026-04-02</v>
       </c>
       <c r="J2" t="str">
-        <v>https://www.1977watches.com</v>
+        <v>https://www.montres1977.com</v>
       </c>
       <c r="K2" t="str">
-        <v/>
+        <v>1977montres</v>
       </c>
       <c r="L2" t="str">
         <v>existing-db</v>
       </c>
       <c r="M2" t="str">
-        <v>French micro-brand based in Paris. Founded 2019. Retro-inspired designs with strong vintage aesthetic. Swiss-assembled. Visitability unconfirmed.</v>
+        <v>French watch brand launched October 2024 (pre-orders) as a standalone spin-off of the Pierre Lannier family watchmaking house, based in Ernolsheim-lès-Saverne, Alsace. Offers two collections — Edmond (classic leather) and Arsène (sporty 904L steel/FKM) — produced in limited annual Millésimes of 99 numbered pieces each, powered by a 100% French France Ébauches automatic caliber and certified Origine France Garantie. Prices range from €1,577–€1,777 (~$1,703–$1,919 USD at ~1.08 EUR/USD).</v>
       </c>
     </row>
     <row r="3">
@@ -510,23 +510,23 @@
       <c r="C3" t="str">
         <v>Budapest, Hungary</v>
       </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
-      <c r="F3" t="str">
-        <v/>
+      <c r="D3">
+        <v>2007</v>
+      </c>
+      <c r="E3">
+        <v>65000</v>
+      </c>
+      <c r="F3">
+        <v>265000</v>
       </c>
       <c r="G3" t="str">
         <v>Active</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>Dignitas Pure "Project XX"</v>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>2026-02-01</v>
       </c>
       <c r="J3" t="str">
         <v>https://www.bexei.hu</v>
@@ -552,34 +552,34 @@
         <v>Paris</v>
       </c>
       <c r="D4">
-        <v>2022</v>
-      </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
-      <c r="F4" t="str">
-        <v/>
+        <v>2024</v>
+      </c>
+      <c r="E4">
+        <v>2430</v>
+      </c>
+      <c r="F4">
+        <v>2700</v>
       </c>
       <c r="G4" t="str">
         <v>Active</v>
       </c>
       <c r="H4" t="str">
-        <v>1712</v>
+        <v>1712 Glaz</v>
       </c>
       <c r="I4" t="str">
-        <v/>
+        <v>2025-04-01</v>
       </c>
       <c r="J4" t="str">
         <v>https://www.abordage-horlogerie.com</v>
       </c>
       <c r="K4" t="str">
-        <v>nobox.nopapers</v>
+        <v>abordage_horlogerie</v>
       </c>
       <c r="L4" t="str">
         <v>existing-db</v>
       </c>
       <c r="M4" t="str">
-        <v>French independent with nautical and sailing heritage. Known for robust field and maritime watches. Based in Paris. Visitability unconfirmed.</v>
+        <v>French microbrand founded in 2024 by two brothers from Saint-Malo, Brittany, inspired by local corsair and maritime heritage. The debut '1712' collection honours privateer René Duguay-Trouin; watches feature guilloche dials, sapphire crystal, and 39mm steel cases water-resistant to 100m. Powered by France Ébauches automatic movements fully manufactured and assembled in France.</v>
       </c>
     </row>
     <row r="5">
@@ -592,23 +592,23 @@
       <c r="C5" t="str">
         <v/>
       </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
-        <v/>
+      <c r="D5">
+        <v>2014</v>
+      </c>
+      <c r="E5">
+        <v>249</v>
+      </c>
+      <c r="F5">
+        <v>599</v>
       </c>
       <c r="G5" t="str">
         <v>Active</v>
       </c>
       <c r="H5" t="str">
-        <v/>
+        <v>Earthrise WWF Partnership Automatic 2025 Edition</v>
       </c>
       <c r="I5" t="str">
-        <v/>
+        <v>2025-04-22</v>
       </c>
       <c r="J5" t="str">
         <v>https://aboutvintage.com</v>
@@ -633,29 +633,29 @@
       <c r="C6" t="str">
         <v/>
       </c>
-      <c r="D6" t="str">
-        <v/>
-      </c>
-      <c r="E6" t="str">
-        <v/>
-      </c>
-      <c r="F6" t="str">
-        <v/>
+      <c r="D6">
+        <v>1931</v>
+      </c>
+      <c r="E6">
+        <v>130</v>
+      </c>
+      <c r="F6">
+        <v>800</v>
       </c>
       <c r="G6" t="str">
         <v>Active</v>
       </c>
       <c r="H6" t="str">
-        <v/>
+        <v>Essence Collection</v>
       </c>
       <c r="I6" t="str">
-        <v/>
+        <v>2025-12-09</v>
       </c>
       <c r="J6" t="str">
         <v>https://adriatica.hr</v>
       </c>
       <c r="K6" t="str">
-        <v/>
+        <v>adriatica_official</v>
       </c>
       <c r="L6" t="str">
         <v>MBWDB</v>
@@ -715,14 +715,14 @@
       <c r="C8" t="str">
         <v/>
       </c>
-      <c r="D8" t="str">
-        <v/>
-      </c>
-      <c r="E8" t="str">
-        <v/>
-      </c>
-      <c r="F8" t="str">
-        <v/>
+      <c r="D8">
+        <v>2013</v>
+      </c>
+      <c r="E8">
+        <v>539</v>
+      </c>
+      <c r="F8">
+        <v>755</v>
       </c>
       <c r="G8" t="str">
         <v>Active</v>
@@ -731,7 +731,7 @@
         <v>Thyïlea GMT</v>
       </c>
       <c r="I8" t="str">
-        <v/>
+        <v>2026-03-30</v>
       </c>
       <c r="J8" t="str">
         <v>https://www.aevig.com</v>
@@ -759,11 +759,11 @@
       <c r="D9">
         <v>1934</v>
       </c>
-      <c r="E9" t="str">
-        <v/>
-      </c>
-      <c r="F9" t="str">
-        <v/>
+      <c r="E9">
+        <v>2214</v>
+      </c>
+      <c r="F9">
+        <v>4158</v>
       </c>
       <c r="G9" t="str">
         <v>Active</v>
@@ -772,7 +772,7 @@
         <v>Type 20 70 ANS</v>
       </c>
       <c r="I9" t="str">
-        <v/>
+        <v>2025-10-23</v>
       </c>
       <c r="J9" t="str">
         <v>https://www.airain.com</v>
@@ -797,29 +797,29 @@
       <c r="C10" t="str">
         <v/>
       </c>
-      <c r="D10" t="str">
-        <v/>
-      </c>
-      <c r="E10" t="str">
-        <v/>
-      </c>
-      <c r="F10" t="str">
-        <v/>
+      <c r="D10">
+        <v>2016</v>
+      </c>
+      <c r="E10">
+        <v>291</v>
+      </c>
+      <c r="F10">
+        <v>526</v>
       </c>
       <c r="G10" t="str">
         <v>Active</v>
       </c>
       <c r="H10" t="str">
-        <v/>
+        <v>Aventyr</v>
       </c>
       <c r="I10" t="str">
-        <v/>
+        <v>2025-12-23</v>
       </c>
       <c r="J10" t="str">
-        <v/>
+        <v>https://akerfalk.se</v>
       </c>
       <c r="K10" t="str">
-        <v/>
+        <v>akerfalk</v>
       </c>
       <c r="L10" t="str">
         <v>MBWDB</v>
@@ -838,8 +838,8 @@
       <c r="C11" t="str">
         <v>Paris</v>
       </c>
-      <c r="D11" t="str">
-        <v/>
+      <c r="D11">
+        <v>2015</v>
       </c>
       <c r="E11">
         <v>549</v>
@@ -854,7 +854,7 @@
         <v>C-02 Baby Héritage Bourbon</v>
       </c>
       <c r="I11" t="str">
-        <v/>
+        <v>2026-03-30</v>
       </c>
       <c r="J11" t="str">
         <v>https://www.akrone.fr</v>
@@ -879,8 +879,8 @@
       <c r="C12" t="str">
         <v>Paris</v>
       </c>
-      <c r="D12" t="str">
-        <v/>
+      <c r="D12">
+        <v>1987</v>
       </c>
       <c r="E12" t="str">
         <v/>
@@ -892,16 +892,16 @@
         <v>Active</v>
       </c>
       <c r="H12" t="str">
-        <v/>
+        <v>MeisterSinger x Alain Silberstein Edition Kaenos (2025 collaboration)</v>
       </c>
       <c r="I12" t="str">
-        <v/>
+        <v>2025-08-08</v>
       </c>
       <c r="J12" t="str">
         <v>https://www.alainsilberstein.com</v>
       </c>
       <c r="K12" t="str">
-        <v/>
+        <v>alainsilbersteinofficial</v>
       </c>
       <c r="L12" t="str">
         <v>existing-db</v>
@@ -920,8 +920,8 @@
       <c r="C13" t="str">
         <v/>
       </c>
-      <c r="D13" t="str">
-        <v/>
+      <c r="D13">
+        <v>2003</v>
       </c>
       <c r="E13">
         <v>1750</v>
@@ -936,7 +936,7 @@
         <v>Kandy Fantasy</v>
       </c>
       <c r="I13" t="str">
-        <v/>
+        <v>2025-12-16</v>
       </c>
       <c r="J13" t="str">
         <v>https://www.alexander-shorokhoff.com</v>
@@ -961,29 +961,29 @@
       <c r="C14" t="str">
         <v>Paris</v>
       </c>
-      <c r="D14" t="str">
-        <v/>
-      </c>
-      <c r="E14" t="str">
-        <v/>
-      </c>
-      <c r="F14" t="str">
-        <v/>
+      <c r="D14">
+        <v>2022</v>
+      </c>
+      <c r="E14">
+        <v>482</v>
+      </c>
+      <c r="F14">
+        <v>540</v>
       </c>
       <c r="G14" t="str">
         <v>Active</v>
       </c>
       <c r="H14" t="str">
-        <v/>
+        <v>L'Odyssée GMT</v>
       </c>
       <c r="I14" t="str">
-        <v/>
+        <v>2026-02-03</v>
       </c>
       <c r="J14" t="str">
         <v>https://www.amaroswatches.com</v>
       </c>
       <c r="K14" t="str">
-        <v/>
+        <v>amaros_watches</v>
       </c>
       <c r="L14" t="str">
         <v>existing-db</v>
@@ -1002,29 +1002,29 @@
       <c r="C15" t="str">
         <v/>
       </c>
-      <c r="D15" t="str">
-        <v/>
-      </c>
-      <c r="E15" t="str">
-        <v/>
-      </c>
-      <c r="F15" t="str">
-        <v/>
+      <c r="D15">
+        <v>2014</v>
+      </c>
+      <c r="E15">
+        <v>1180</v>
+      </c>
+      <c r="F15">
+        <v>2180</v>
       </c>
       <c r="G15" t="str">
         <v>Active</v>
       </c>
       <c r="H15" t="str">
-        <v/>
+        <v>OCEANMASTER II 1000M</v>
       </c>
       <c r="I15" t="str">
-        <v/>
+        <v>2023-04-12</v>
       </c>
       <c r="J15" t="str">
         <v>https://andersmann-watches.com</v>
       </c>
       <c r="K15" t="str">
-        <v/>
+        <v>andersmannwatch</v>
       </c>
       <c r="L15" t="str">
         <v>MBWDB</v>
@@ -1043,14 +1043,14 @@
       <c r="C16" t="str">
         <v/>
       </c>
-      <c r="D16" t="str">
-        <v/>
-      </c>
-      <c r="E16" t="str">
-        <v/>
-      </c>
-      <c r="F16" t="str">
-        <v/>
+      <c r="D16">
+        <v>1997</v>
+      </c>
+      <c r="E16">
+        <v>2951</v>
+      </c>
+      <c r="F16">
+        <v>5113</v>
       </c>
       <c r="G16" t="str">
         <v>Active</v>
@@ -1059,7 +1059,7 @@
         <v>Nautilo Vintage Green</v>
       </c>
       <c r="I16" t="str">
-        <v/>
+        <v>2025-03-20</v>
       </c>
       <c r="J16" t="str">
         <v>https://www.anonimo.com</v>
@@ -1084,14 +1084,14 @@
       <c r="C17" t="str">
         <v>Glasgow, Scotland</v>
       </c>
-      <c r="D17" t="str">
-        <v/>
-      </c>
-      <c r="E17" t="str">
-        <v/>
-      </c>
-      <c r="F17" t="str">
-        <v/>
+      <c r="D17">
+        <v>2016</v>
+      </c>
+      <c r="E17">
+        <v>2255</v>
+      </c>
+      <c r="F17">
+        <v>4656</v>
       </c>
       <c r="G17" t="str">
         <v>Active</v>
@@ -1100,7 +1100,7 @@
         <v>Model 2 Porcelain</v>
       </c>
       <c r="I17" t="str">
-        <v/>
+        <v>2025-05-29</v>
       </c>
       <c r="J17" t="str">
         <v>https://anordain.com</v>
@@ -1248,14 +1248,14 @@
       <c r="C21" t="str">
         <v>Paris</v>
       </c>
-      <c r="D21" t="str">
-        <v/>
+      <c r="D21">
+        <v>2022</v>
       </c>
       <c r="E21">
         <v>995</v>
       </c>
-      <c r="F21" t="str">
-        <v/>
+      <c r="F21">
+        <v>1075</v>
       </c>
       <c r="G21" t="str">
         <v>Active</v>
@@ -1264,13 +1264,13 @@
         <v>SPEED</v>
       </c>
       <c r="I21" t="str">
-        <v/>
+        <v>2026-02-09</v>
       </c>
       <c r="J21" t="str">
         <v>https://www.aquilonandco.com</v>
       </c>
       <c r="K21" t="str">
-        <v/>
+        <v>aquilonandco</v>
       </c>
       <c r="L21" t="str">
         <v>existing-db</v>
@@ -1289,29 +1289,29 @@
       <c r="C22" t="str">
         <v>Frederiksberg, Denmark</v>
       </c>
-      <c r="D22" t="str">
-        <v/>
-      </c>
-      <c r="E22" t="str">
-        <v/>
-      </c>
-      <c r="F22" t="str">
-        <v/>
+      <c r="D22">
+        <v>2018</v>
+      </c>
+      <c r="E22">
+        <v>3950</v>
+      </c>
+      <c r="F22">
+        <v>5450</v>
       </c>
       <c r="G22" t="str">
         <v>Active</v>
       </c>
       <c r="H22" t="str">
-        <v/>
+        <v>ARC II – D'Arc Sh'Arc</v>
       </c>
       <c r="I22" t="str">
-        <v/>
+        <v>2025-08-01</v>
       </c>
       <c r="J22" t="str">
         <v>https://www.arcanaut.dk</v>
       </c>
       <c r="K22" t="str">
-        <v/>
+        <v>arcanaut_watches</v>
       </c>
       <c r="L22" t="str">
         <v>existing-db</v>

</xml_diff>

<commit_message>
data: clear dead URLs and re-source via Brave Search
- check-websites.js identified 282 dead domains across all regions
- Cleared 19 dead URLs (hostname-matched against live check results)
- Re-ran find-websites-brave.js: 59/60 replacement URLs found
- Spreadsheet rebuilt

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/watch-microbrand-database.xlsx
+++ b/watch-microbrand-database.xlsx
@@ -652,7 +652,7 @@
         <v>2025-12-09</v>
       </c>
       <c r="J6" t="str">
-        <v>https://adriatica.hr</v>
+        <v>https://adriaticawatches.ch/en/</v>
       </c>
       <c r="K6" t="str">
         <v>adriatica_official</v>
@@ -1226,7 +1226,7 @@
         <v/>
       </c>
       <c r="J20" t="str">
-        <v/>
+        <v>https://aquastar.ch/</v>
       </c>
       <c r="K20" t="str">
         <v/>
@@ -1595,7 +1595,7 @@
         <v/>
       </c>
       <c r="J29" t="str">
-        <v/>
+        <v>https://augustberg.com/</v>
       </c>
       <c r="K29" t="str">
         <v/>
@@ -1923,7 +1923,7 @@
         <v/>
       </c>
       <c r="J37" t="str">
-        <v>https://ballast-watch.de</v>
+        <v>https://www.ballast1903.com/</v>
       </c>
       <c r="K37" t="str">
         <v/>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="J42" t="str">
-        <v/>
+        <v>https://www.batavi-watches.com/</v>
       </c>
       <c r="K42" t="str">
         <v/>
@@ -2210,7 +2210,7 @@
         <v/>
       </c>
       <c r="J44" t="str">
-        <v>https://bausele.de</v>
+        <v>https://www.bausele.com/</v>
       </c>
       <c r="K44" t="str">
         <v>bausele_watches</v>
@@ -3768,7 +3768,7 @@
         <v/>
       </c>
       <c r="J82" t="str">
-        <v/>
+        <v>https://dingemansmechanischehorloges.nl/</v>
       </c>
       <c r="K82" t="str">
         <v/>
@@ -4055,7 +4055,7 @@
         <v/>
       </c>
       <c r="J89" t="str">
-        <v/>
+        <v>https://www.delftwatchworks.com/en/</v>
       </c>
       <c r="K89" t="str">
         <v/>
@@ -4137,7 +4137,7 @@
         <v/>
       </c>
       <c r="J91" t="str">
-        <v/>
+        <v>https://dennisonwatch.com/</v>
       </c>
       <c r="K91" t="str">
         <v/>
@@ -4588,7 +4588,7 @@
         <v/>
       </c>
       <c r="J102" t="str">
-        <v/>
+        <v>https://draytonwatches.com/</v>
       </c>
       <c r="K102" t="str">
         <v/>
@@ -5080,7 +5080,7 @@
         <v/>
       </c>
       <c r="J114" t="str">
-        <v/>
+        <v>http://www.enicar.com/</v>
       </c>
       <c r="K114" t="str">
         <v/>
@@ -5695,7 +5695,7 @@
         <v/>
       </c>
       <c r="J129" t="str">
-        <v/>
+        <v>https://www.guinand-uhren.de/home-en.html</v>
       </c>
       <c r="K129" t="str">
         <v/>
@@ -6228,7 +6228,7 @@
         <v/>
       </c>
       <c r="J142" t="str">
-        <v/>
+        <v>https://www.humbert-droz.fr/en/</v>
       </c>
       <c r="K142" t="str">
         <v/>
@@ -6597,7 +6597,7 @@
         <v/>
       </c>
       <c r="J151" t="str">
-        <v/>
+        <v>https://mccabewatches.com/</v>
       </c>
       <c r="K151" t="str">
         <v/>
@@ -6925,7 +6925,7 @@
         <v/>
       </c>
       <c r="J159" t="str">
-        <v/>
+        <v>https://www.karlskronawatch.com/</v>
       </c>
       <c r="K159" t="str">
         <v/>
@@ -7458,7 +7458,7 @@
         <v/>
       </c>
       <c r="J172" t="str">
-        <v/>
+        <v>https://www.lang-und-heyne.de/en/collection/</v>
       </c>
       <c r="K172" t="str">
         <v/>
@@ -7499,7 +7499,7 @@
         <v/>
       </c>
       <c r="J173" t="str">
-        <v/>
+        <v>https://apelvikenwatches.com/pages/about</v>
       </c>
       <c r="K173" t="str">
         <v/>
@@ -8196,7 +8196,7 @@
         <v/>
       </c>
       <c r="J190" t="str">
-        <v/>
+        <v>https://marketplace.watchcharts.com/listings/brand/manchester+watch+works</v>
       </c>
       <c r="K190" t="str">
         <v/>
@@ -8278,7 +8278,7 @@
         <v/>
       </c>
       <c r="J192" t="str">
-        <v/>
+        <v>https://www.marcdarno.com</v>
       </c>
       <c r="K192" t="str">
         <v/>
@@ -8770,7 +8770,7 @@
         <v/>
       </c>
       <c r="J204" t="str">
-        <v/>
+        <v>https://www.merkurwatch.com/</v>
       </c>
       <c r="K204" t="str">
         <v/>
@@ -8811,7 +8811,7 @@
         <v/>
       </c>
       <c r="J205" t="str">
-        <v/>
+        <v>https://miangcopenhagen.com/pages/about-us</v>
       </c>
       <c r="K205" t="str">
         <v/>
@@ -8934,7 +8934,7 @@
         <v/>
       </c>
       <c r="J208" t="str">
-        <v/>
+        <v>https://bulangandsons.com/collections/minerva</v>
       </c>
       <c r="K208" t="str">
         <v/>
@@ -9344,7 +9344,7 @@
         <v/>
       </c>
       <c r="J218" t="str">
-        <v>https://www.nordgreen.io</v>
+        <v>https://nordgreen.com/en-us</v>
       </c>
       <c r="K218" t="str">
         <v>nordgreenofficial</v>
@@ -9590,7 +9590,7 @@
         <v/>
       </c>
       <c r="J224" t="str">
-        <v/>
+        <v>https://www.orologicalamai.com/</v>
       </c>
       <c r="K224" t="str">
         <v/>
@@ -9754,7 +9754,7 @@
         <v/>
       </c>
       <c r="J228" t="str">
-        <v/>
+        <v>https://pinet-montrivel.com/en/1729-2/</v>
       </c>
       <c r="K228" t="str">
         <v/>
@@ -10123,7 +10123,7 @@
         <v/>
       </c>
       <c r="J237" t="str">
-        <v/>
+        <v>https://radiuminstruments.no/</v>
       </c>
       <c r="K237" t="str">
         <v/>
@@ -11025,7 +11025,7 @@
         <v>2024-09-15</v>
       </c>
       <c r="J259" t="str">
-        <v>https://www.serica.watches</v>
+        <v>https://serica-watches.com/en</v>
       </c>
       <c r="K259" t="str">
         <v>serica_watches</v>
@@ -11394,7 +11394,7 @@
         <v/>
       </c>
       <c r="J268" t="str">
-        <v/>
+        <v>https://www.stefanobragawatches.com/products/selene-dlc</v>
       </c>
       <c r="K268" t="str">
         <v/>
@@ -11927,7 +11927,7 @@
         <v/>
       </c>
       <c r="J281" t="str">
-        <v/>
+        <v>http://www.tmfwatches.com/en/</v>
       </c>
       <c r="K281" t="str">
         <v/>
@@ -12091,7 +12091,7 @@
         <v/>
       </c>
       <c r="J285" t="str">
-        <v>https://www.tufina.de</v>
+        <v>https://tufinawatches.com/</v>
       </c>
       <c r="K285" t="str">
         <v/>
@@ -12296,7 +12296,7 @@
         <v/>
       </c>
       <c r="J290" t="str">
-        <v/>
+        <v>https://ugolinimeccanicawatches.com/</v>
       </c>
       <c r="K290" t="str">
         <v/>
@@ -12419,7 +12419,7 @@
         <v/>
       </c>
       <c r="J293" t="str">
-        <v/>
+        <v>https://www.valhallaofnorway.no/</v>
       </c>
       <c r="K293" t="str">
         <v/>
@@ -15028,7 +15028,7 @@
         <v/>
       </c>
       <c r="J46" t="str">
-        <v/>
+        <v>https://grandeur-usa.com/</v>
       </c>
       <c r="K46" t="str">
         <v/>
@@ -16340,7 +16340,7 @@
         <v/>
       </c>
       <c r="J78" t="str">
-        <v/>
+        <v>https://rarebirds.de/</v>
       </c>
       <c r="K78" t="str">
         <v/>
@@ -17760,7 +17760,7 @@
         <v/>
       </c>
       <c r="J9" t="str">
-        <v/>
+        <v>https://bureiwatches.com/</v>
       </c>
       <c r="K9" t="str">
         <v/>
@@ -17842,7 +17842,7 @@
         <v/>
       </c>
       <c r="J11" t="str">
-        <v/>
+        <v>https://linkandtag.com/2025/10/18/ckl-watches/</v>
       </c>
       <c r="K11" t="str">
         <v/>
@@ -17883,7 +17883,7 @@
         <v/>
       </c>
       <c r="J12" t="str">
-        <v/>
+        <v>https://corgeutwatchco.com/</v>
       </c>
       <c r="K12" t="str">
         <v/>
@@ -17924,7 +17924,7 @@
         <v/>
       </c>
       <c r="J13" t="str">
-        <v/>
+        <v>https://crrju.com/</v>
       </c>
       <c r="K13" t="str">
         <v/>
@@ -18047,7 +18047,7 @@
         <v/>
       </c>
       <c r="J16" t="str">
-        <v/>
+        <v>https://guanqin-watch.com/</v>
       </c>
       <c r="K16" t="str">
         <v/>
@@ -18211,7 +18211,7 @@
         <v/>
       </c>
       <c r="J20" t="str">
-        <v/>
+        <v>https://jaipur.watch/en-us</v>
       </c>
       <c r="K20" t="str">
         <v/>
@@ -18252,7 +18252,7 @@
         <v/>
       </c>
       <c r="J21" t="str">
-        <v>https://www.kentex.jp</v>
+        <v>http://www.kentexwatch.com/</v>
       </c>
       <c r="K21" t="str">
         <v>kentex_official</v>
@@ -18293,7 +18293,7 @@
         <v/>
       </c>
       <c r="J22" t="str">
-        <v/>
+        <v>https://kiwametokyo.com/en/collections/watches</v>
       </c>
       <c r="K22" t="str">
         <v/>
@@ -18703,7 +18703,7 @@
         <v/>
       </c>
       <c r="J32" t="str">
-        <v/>
+        <v>https://www.pitzmann.com/</v>
       </c>
       <c r="K32" t="str">
         <v/>
@@ -18744,7 +18744,7 @@
         <v/>
       </c>
       <c r="J33" t="str">
-        <v/>
+        <v>https://sugesswatch.com/</v>
       </c>
       <c r="K33" t="str">
         <v/>
@@ -18867,7 +18867,7 @@
         <v/>
       </c>
       <c r="J36" t="str">
-        <v/>
+        <v>https://solvil-et-titus.sg/</v>
       </c>
       <c r="K36" t="str">
         <v/>
@@ -18908,7 +18908,7 @@
         <v/>
       </c>
       <c r="J37" t="str">
-        <v/>
+        <v>https://wancherwatch.com/</v>
       </c>
       <c r="K37" t="str">
         <v/>
@@ -24346,7 +24346,7 @@
         <v/>
       </c>
       <c r="J128" t="str">
-        <v/>
+        <v>https://poshmark.com/brand/charles%20Delon-Women-Accessories-Watches</v>
       </c>
       <c r="K128" t="str">
         <v/>
@@ -25863,7 +25863,7 @@
         <v/>
       </c>
       <c r="J165" t="str">
-        <v>https://diakka.co/</v>
+        <v>https://shop.simon.com/collections/curated-watches-and-sunglasses?Brand=Diakka</v>
       </c>
       <c r="K165" t="str">
         <v/>
@@ -27913,7 +27913,7 @@
         <v/>
       </c>
       <c r="J215" t="str">
-        <v>https://www.eza.watch</v>
+        <v>https://ezawatches.com/</v>
       </c>
       <c r="K215" t="str">
         <v/>
@@ -29512,7 +29512,7 @@
         <v/>
       </c>
       <c r="J254" t="str">
-        <v>https://www.gerlach.watch</v>
+        <v>https://www.gerlach.org.pl/en/g-gerlach/</v>
       </c>
       <c r="K254" t="str">
         <v/>
@@ -30373,7 +30373,7 @@
         <v/>
       </c>
       <c r="J275" t="str">
-        <v>https://www.h2owatches.dk</v>
+        <v>https://www.h2o-watch.com/</v>
       </c>
       <c r="K275" t="str">
         <v>h2owatches</v>
@@ -32956,7 +32956,7 @@
         <v/>
       </c>
       <c r="J338" t="str">
-        <v>https://www.jswatchco.is</v>
+        <v>https://www.jswatch.com</v>
       </c>
       <c r="K338" t="str">
         <v/>
@@ -33571,7 +33571,7 @@
         <v/>
       </c>
       <c r="J353" t="str">
-        <v>https://www.kuoe.jp</v>
+        <v>https://www.kuoe-en.com/</v>
       </c>
       <c r="K353" t="str">
         <v/>
@@ -42960,7 +42960,7 @@
         <v/>
       </c>
       <c r="J582" t="str">
-        <v>https://www.riskers.co</v>
+        <v>https://riskers-watches.com/</v>
       </c>
       <c r="K582" t="str">
         <v/>

</xml_diff>

<commit_message>
chore: rebuild spreadsheet after discover-brands run (229 lastActivityDate updates)
</commit_message>
<xml_diff>
--- a/watch-microbrand-database.xlsx
+++ b/watch-microbrand-database.xlsx
@@ -608,7 +608,7 @@
         <v>NIMROD</v>
       </c>
       <c r="I5" t="str">
-        <v>2025-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J5" t="str">
         <v>https://www.abingerwatches.com</v>
@@ -895,7 +895,7 @@
         <v>Thyïlea GMT</v>
       </c>
       <c r="I12" t="str">
-        <v>2026-03-30</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J12" t="str">
         <v>https://www.aevig.com</v>
@@ -977,7 +977,7 @@
         <v>Type 20 70 ANS</v>
       </c>
       <c r="I14" t="str">
-        <v>2025-10-23</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J14" t="str">
         <v>https://www.airain.com</v>
@@ -1182,7 +1182,7 @@
         <v/>
       </c>
       <c r="I19" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J19" t="str">
         <v>https://www.alato.se/en</v>
@@ -1264,7 +1264,7 @@
         <v>A3 Omen II</v>
       </c>
       <c r="I21" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J21" t="str">
         <v>https://alexanderjameswatches.com/</v>
@@ -1305,7 +1305,7 @@
         <v>Kandy Fantasy</v>
       </c>
       <c r="I22" t="str">
-        <v>2025-12-16</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J22" t="str">
         <v>https://www.alexander-shorokhoff.com</v>
@@ -1387,7 +1387,7 @@
         <v>Model Three Diver</v>
       </c>
       <c r="I24" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J24" t="str">
         <v>https://alkinwatches.com/</v>
@@ -1551,7 +1551,7 @@
         <v>Nautilo Vintage Green</v>
       </c>
       <c r="I28" t="str">
-        <v>2022-11-14</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J28" t="str">
         <v>https://www.anonimo.com</v>
@@ -1592,7 +1592,7 @@
         <v>Model 2 Porcelain</v>
       </c>
       <c r="I29" t="str">
-        <v>2025-05-29</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J29" t="str">
         <v>https://anordain.com</v>
@@ -1879,7 +1879,7 @@
         <v>Klassik 200</v>
       </c>
       <c r="I36" t="str">
-        <v>2024-12-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J36" t="str">
         <v>https://www.archimede-watches.com</v>
@@ -1920,7 +1920,7 @@
         <v>Aquaristo Automatic 4H98294 (Klassik Diver series)</v>
       </c>
       <c r="I37" t="str">
-        <v>2026-02-23</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J37" t="str">
         <v>https://www.aristo.de</v>
@@ -2084,7 +2084,7 @@
         <v>FL 1889</v>
       </c>
       <c r="I41" t="str">
-        <v>2025-11-04</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J41" t="str">
         <v>https://www.ateliercaradant.com</v>
@@ -2576,7 +2576,7 @@
         <v>Chapter 8</v>
       </c>
       <c r="I53" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J53" t="str">
         <v>https://www.ba111od.com</v>
@@ -2781,7 +2781,7 @@
         <v>Aquascaphe</v>
       </c>
       <c r="I58" t="str">
-        <v>2024-10-15</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J58" t="str">
         <v>https://www.balticwatches.com</v>
@@ -2986,7 +2986,7 @@
         <v/>
       </c>
       <c r="I63" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J63" t="str">
         <v>https://www.bausele.com/</v>
@@ -3027,7 +3027,7 @@
         <v/>
       </c>
       <c r="I64" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J64" t="str">
         <v>https://www.beaubleu.fr</v>
@@ -3068,7 +3068,7 @@
         <v>Element 39.5mm</v>
       </c>
       <c r="I65" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J65" t="str">
         <v>https://beaucroftwatches.com/</v>
@@ -3150,7 +3150,7 @@
         <v>Rotary (2025)</v>
       </c>
       <c r="I67" t="str">
-        <v>2025-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J67" t="str">
         <v>https://www.behrenswatches.com</v>
@@ -3970,7 +3970,7 @@
         <v/>
       </c>
       <c r="I87" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J87" t="str">
         <v>https://www.bravur.com</v>
@@ -4052,7 +4052,7 @@
         <v>Terra Nova Jumping Hour</v>
       </c>
       <c r="I89" t="str">
-        <v>2024-10-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J89" t="str">
         <v>https://www.bremont.com</v>
@@ -4339,7 +4339,7 @@
         <v/>
       </c>
       <c r="I96" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J96" t="str">
         <v>https://www.bruvik.com</v>
@@ -4626,7 +4626,7 @@
         <v/>
       </c>
       <c r="I103" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J103" t="str">
         <v>https://www.cadola.ch</v>
@@ -5036,7 +5036,7 @@
         <v>C60 Trident Pro</v>
       </c>
       <c r="I113" t="str">
-        <v>2024-10-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J113" t="str">
         <v>https://www.christopherward.com</v>
@@ -5200,7 +5200,7 @@
         <v/>
       </c>
       <c r="I117" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J117" t="str">
         <v>https://www.circula.com</v>
@@ -5282,7 +5282,7 @@
         <v>Photic MKII</v>
       </c>
       <c r="I119" t="str">
-        <v>2024-12-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J119" t="str">
         <v>https://www.clemencewatches.com/</v>
@@ -5364,7 +5364,7 @@
         <v/>
       </c>
       <c r="I121" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J121" t="str">
         <v>https://www.code41.com</v>
@@ -5979,7 +5979,7 @@
         <v>DA47</v>
       </c>
       <c r="I136" t="str">
-        <v>2024-10-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J136" t="str">
         <v>https://www.damasko.de</v>
@@ -6061,7 +6061,7 @@
         <v>Argonautic World Traveller</v>
       </c>
       <c r="I138" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J138" t="str">
         <v>https://www.davosa.com</v>
@@ -6225,7 +6225,7 @@
         <v>DEKLA Pilot Watch 40mm Type B Bronze CuSn8</v>
       </c>
       <c r="I142" t="str">
-        <v>2024-12-31</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J142" t="str">
         <v>https://deklawatches.com/en</v>
@@ -6389,7 +6389,7 @@
         <v/>
       </c>
       <c r="I146" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J146" t="str">
         <v>https://dennisonwatch.com/</v>
@@ -6471,7 +6471,7 @@
         <v/>
       </c>
       <c r="I148" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J148" t="str">
         <v>https://www.depancel.com</v>
@@ -7004,7 +7004,7 @@
         <v/>
       </c>
       <c r="I161" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J161" t="str">
         <v>https://www.doxawatch.com</v>
@@ -7250,7 +7250,7 @@
         <v/>
       </c>
       <c r="I167" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J167" t="str">
         <v>https://www.dufa.com</v>
@@ -7414,7 +7414,7 @@
         <v>Rivanera</v>
       </c>
       <c r="I171" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J171" t="str">
         <v>https://www.echoneutra.com</v>
@@ -7701,7 +7701,7 @@
         <v>Arinis</v>
       </c>
       <c r="I178" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J178" t="str">
         <v>https://www.elkawatch.ch/</v>
@@ -8111,7 +8111,7 @@
         <v>Light Racing Range</v>
       </c>
       <c r="I188" t="str">
-        <v>2026-01-21</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J188" t="str">
         <v>https://www.eskawatches.com/en</v>
@@ -8193,7 +8193,7 @@
         <v/>
       </c>
       <c r="I190" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J190" t="str">
         <v>https://ezawatches.com/</v>
@@ -8234,7 +8234,7 @@
         <v>35mm Cushion Case Collection</v>
       </c>
       <c r="I191" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J191" t="str">
         <v>https://www.farer.co.uk</v>
@@ -8275,7 +8275,7 @@
         <v>Nexus</v>
       </c>
       <c r="I192" t="str">
-        <v>2024-12-19</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J192" t="str">
         <v>https://fatherswatches.com/en</v>
@@ -8398,7 +8398,7 @@
         <v>Brunswick</v>
       </c>
       <c r="I195" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J195" t="str">
         <v>https://www.fearswatches.com</v>
@@ -8439,7 +8439,7 @@
         <v>NAUTICMASTER FIELD DIVER</v>
       </c>
       <c r="I196" t="str">
-        <v>2025-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J196" t="str">
         <v>https://www.findeisen-uhren.com/en</v>
@@ -8644,7 +8644,7 @@
         <v>Essence Ceramica GT</v>
       </c>
       <c r="I201" t="str">
-        <v>2024-12-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J201" t="str">
         <v>https://www.formexwatch.com</v>
@@ -8685,7 +8685,7 @@
         <v>Abyss</v>
       </c>
       <c r="I202" t="str">
-        <v>2024-10-15</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J202" t="str">
         <v>https://www.fortis-watches.com</v>
@@ -8808,7 +8808,7 @@
         <v>Disco Onyx Diamonds</v>
       </c>
       <c r="I205" t="str">
-        <v>2024-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J205" t="str">
         <v>https://www.furlanmarri.com</v>
@@ -9013,7 +9013,7 @@
         <v>Pioneer</v>
       </c>
       <c r="I210" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J210" t="str">
         <v>https://www.geckota.com</v>
@@ -9300,7 +9300,7 @@
         <v>Aquareef 40</v>
       </c>
       <c r="I217" t="str">
-        <v>2025-09-15</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J217" t="str">
         <v>https://www.golbywatches.co.uk</v>
@@ -9874,7 +9874,7 @@
         <v>Sport</v>
       </c>
       <c r="I231" t="str">
-        <v>2024-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J231" t="str">
         <v>https://www.hagleywest.com</v>
@@ -10161,7 +10161,7 @@
         <v>Radiance</v>
       </c>
       <c r="I238" t="str">
-        <v>2024-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J238" t="str">
         <v>https://heinrich.watch/en-us</v>
@@ -10243,7 +10243,7 @@
         <v/>
       </c>
       <c r="I240" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J240" t="str">
         <v>https://www.henryarcherwatches.com</v>
@@ -10325,7 +10325,7 @@
         <v>Marinor Classic</v>
       </c>
       <c r="I242" t="str">
-        <v>2024-10-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J242" t="str">
         <v>https://www.heronwatches.com/</v>
@@ -10448,7 +10448,7 @@
         <v>SIGNATURE ORNAMENT</v>
       </c>
       <c r="I245" t="str">
-        <v>2025</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J245" t="str">
         <v>https://www.holthinrichs.com</v>
@@ -10489,7 +10489,7 @@
         <v>K-TMR Micro-Rotor Tourbillon</v>
       </c>
       <c r="I246" t="str">
-        <v>2024-07-24</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J246" t="str">
         <v>https://www.horage.com</v>
@@ -10694,7 +10694,7 @@
         <v>Horopod</v>
       </c>
       <c r="I251" t="str">
-        <v>2025-01-08</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J251" t="str">
         <v>https://www.ikepod.com</v>
@@ -10899,7 +10899,7 @@
         <v/>
       </c>
       <c r="I256" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J256" t="str">
         <v>https://www.isotopewatches.com</v>
@@ -11309,7 +11309,7 @@
         <v/>
       </c>
       <c r="I266" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J266" t="str">
         <v>https://www.jswatch.com</v>
@@ -11350,7 +11350,7 @@
         <v>Aquaris Diver</v>
       </c>
       <c r="I267" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J267" t="str">
         <v>https://www.junghans.de</v>
@@ -11842,7 +11842,7 @@
         <v>Klok-01 5th Anniversary</v>
       </c>
       <c r="I279" t="str">
-        <v>2024-10-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J279" t="str">
         <v>https://www.klokers.com</v>
@@ -11965,7 +11965,7 @@
         <v>Projekt 02 Variant B</v>
       </c>
       <c r="I282" t="str">
-        <v>2024-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J282" t="str">
         <v>https://kollokium.com/</v>
@@ -12170,7 +12170,7 @@
         <v>Laco Köln</v>
       </c>
       <c r="I287" t="str">
-        <v>2024-12-19</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J287" t="str">
         <v>https://www.laco.de</v>
@@ -12416,7 +12416,7 @@
         <v/>
       </c>
       <c r="I293" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J293" t="str">
         <v>https://www.laventure.ch</v>
@@ -12867,7 +12867,7 @@
         <v>Model No.2 Chronograph</v>
       </c>
       <c r="I304" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J304" t="str">
         <v>https://www.lorcawatches.com</v>
@@ -12908,7 +12908,7 @@
         <v>LS06</v>
       </c>
       <c r="I305" t="str">
-        <v>2024-12-31</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J305" t="str">
         <v>https://loresum.watch/collections/all-products</v>
@@ -13236,7 +13236,7 @@
         <v>Hudson 38 MK5</v>
       </c>
       <c r="I313" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J313" t="str">
         <v>https://www.maenwatches.com</v>
@@ -13523,7 +13523,7 @@
         <v/>
       </c>
       <c r="I320" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J320" t="str">
         <v>https://www.marc-and-sons.com</v>
@@ -13892,7 +13892,7 @@
         <v>Dark Surge 300A (Adriatic)</v>
       </c>
       <c r="I329" t="str">
-        <v>2025-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J329" t="str">
         <v>https://www.marnaut.com</v>
@@ -14261,7 +14261,7 @@
         <v>PROSPERITY GMT SNOWY OWL</v>
       </c>
       <c r="I338" t="str">
-        <v>2025-08-25</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J338" t="str">
         <v>https://www.maystonewatches.com/</v>
@@ -14343,7 +14343,7 @@
         <v>C1</v>
       </c>
       <c r="I340" t="str">
-        <v>2025-11-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J340" t="str">
         <v>https://mcquaide.co.uk/</v>
@@ -14753,7 +14753,7 @@
         <v>Milgraph T5 Pilot Series Worldtimer</v>
       </c>
       <c r="I350" t="str">
-        <v>2025-08-14</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J350" t="str">
         <v>https://www.micromilspec.com</v>
@@ -15450,7 +15450,7 @@
         <v>Daydreamer</v>
       </c>
       <c r="I367" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J367" t="str">
         <v>https://www.mrjoneswatches.com</v>
@@ -15573,7 +15573,7 @@
         <v>Diver II Automatic</v>
       </c>
       <c r="I370" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J370" t="str">
         <v>https://nautage.com/</v>
@@ -15614,7 +15614,7 @@
         <v>LM02 Type C</v>
       </c>
       <c r="I371" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J371" t="str">
         <v>https://www.neotypewatches.com</v>
@@ -15737,7 +15737,7 @@
         <v>6BB NP Professional Chronograph</v>
       </c>
       <c r="I374" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J374" t="str">
         <v>https://newmarkwatchcompany.com/</v>
@@ -15901,7 +15901,7 @@
         <v>F77 SST GREEN AVENTURINE MK2</v>
       </c>
       <c r="I378" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J378" t="str">
         <v>https://www.nivadagrenchenofficial.com</v>
@@ -16024,7 +16024,7 @@
         <v>The Brú 750</v>
       </c>
       <c r="I381" t="str">
-        <v>2026-03-20</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J381" t="str">
         <v>https://nomadicwatches.com/en-us</v>
@@ -16844,7 +16844,7 @@
         <v>Sector</v>
       </c>
       <c r="I401" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J401" t="str">
         <v>https://www.pareawatches.com</v>
@@ -16926,7 +16926,7 @@
         <v>Neo Collection</v>
       </c>
       <c r="I403" t="str">
-        <v>2026-03-23</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J403" t="str">
         <v>https://www.paulinwatches.com</v>
@@ -16967,7 +16967,7 @@
         <v>Final Frontier</v>
       </c>
       <c r="I404" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J404" t="str">
         <v>https://www.pedral.eu/</v>
@@ -17213,7 +17213,7 @@
         <v>Pure</v>
       </c>
       <c r="I410" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J410" t="str">
         <v>https://www.pinionwatches.com</v>
@@ -17664,7 +17664,7 @@
         <v>L'INSTANT SONORE</v>
       </c>
       <c r="I421" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J421" t="str">
         <v>https://www.radcliffewatches.com</v>
@@ -18156,7 +18156,7 @@
         <v/>
       </c>
       <c r="I433" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J433" t="str">
         <v>https://www.revue-thommen.com</v>
@@ -18853,7 +18853,7 @@
         <v/>
       </c>
       <c r="I450" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J450" t="str">
         <v>https://www.sangin-instruments.com</v>
@@ -18894,7 +18894,7 @@
         <v/>
       </c>
       <c r="I451" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J451" t="str">
         <v>https://www.sartorybillard.com</v>
@@ -19017,7 +19017,7 @@
         <v>The GMT</v>
       </c>
       <c r="I454" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J454" t="str">
         <v>https://www.schofieldwatches.com</v>
@@ -19099,7 +19099,7 @@
         <v>Diver One D1-500</v>
       </c>
       <c r="I456" t="str">
-        <v>2026-03-06</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J456" t="str">
         <v>https://www.scurfawatches.com</v>
@@ -19263,7 +19263,7 @@
         <v>M1 Moonphase</v>
       </c>
       <c r="I460" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J460" t="str">
         <v>https://seltenwatch.com/</v>
@@ -19386,7 +19386,7 @@
         <v>Serica Field Watch</v>
       </c>
       <c r="I463" t="str">
-        <v>2024-09-15</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J463" t="str">
         <v>https://serica-watches.com/en</v>
@@ -19591,7 +19591,7 @@
         <v/>
       </c>
       <c r="I468" t="str">
-        <v>2024-10-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J468" t="str">
         <v>https://www.sinn.de</v>
@@ -19960,7 +19960,7 @@
         <v/>
       </c>
       <c r="I477" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J477" t="str">
         <v>https://www.spaceone-watches.com</v>
@@ -20042,7 +20042,7 @@
         <v>Squale Matic S</v>
       </c>
       <c r="I479" t="str">
-        <v>2024-12-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J479" t="str">
         <v>https://www.squalewatches.com</v>
@@ -20206,7 +20206,7 @@
         <v>Marus 2.0 Edition Küste</v>
       </c>
       <c r="I483" t="str">
-        <v>2025-12-03</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J483" t="str">
         <v>https://www.sternglas.com</v>
@@ -20288,7 +20288,7 @@
         <v>Chrono Black Forest Moon</v>
       </c>
       <c r="I485" t="str">
-        <v>2024-11-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J485" t="str">
         <v>https://www.stowa.de</v>
@@ -20329,7 +20329,7 @@
         <v/>
       </c>
       <c r="I486" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J486" t="str">
         <v>https://straumwatches.com</v>
@@ -20534,7 +20534,7 @@
         <v/>
       </c>
       <c r="I491" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J491" t="str">
         <v>https://www.studiounderd0g.com</v>
@@ -20739,7 +20739,7 @@
         <v>Cannonball GMT</v>
       </c>
       <c r="I496" t="str">
-        <v>2024-12-31</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J496" t="str">
         <v>https://www.syewatches.com</v>
@@ -21026,7 +21026,7 @@
         <v/>
       </c>
       <c r="I503" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J503" t="str">
         <v>https://www.terraCielomare.com</v>
@@ -21149,7 +21149,7 @@
         <v>Smiths Commander 71 PRS-71</v>
       </c>
       <c r="I506" t="str">
-        <v>2026-03-10</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J506" t="str">
         <v>https://www.timefactors.com</v>
@@ -21354,7 +21354,7 @@
         <v>Marine Automatik 37mm</v>
       </c>
       <c r="I511" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J511" t="str">
         <v>https://www.tourby.de</v>
@@ -21436,7 +21436,7 @@
         <v>1000M</v>
       </c>
       <c r="I513" t="str">
-        <v>2024-06-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J513" t="str">
         <v>https://www.trematic.de</v>
@@ -21600,7 +21600,7 @@
         <v/>
       </c>
       <c r="I517" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J517" t="str">
         <v>https://tufinawatches.com/</v>
@@ -21641,7 +21641,7 @@
         <v>Shellback V2</v>
       </c>
       <c r="I518" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J518" t="str">
         <v>https://www.tuseno.com</v>
@@ -21805,7 +21805,7 @@
         <v>TREK DUAL SERIES 01</v>
       </c>
       <c r="I522" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J522" t="str">
         <v>https://www.ubiqwatches.com</v>
@@ -21928,7 +21928,7 @@
         <v/>
       </c>
       <c r="I525" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J525" t="str">
         <v>https://www.undonewatches.com</v>
@@ -21969,7 +21969,7 @@
         <v>Modello Tre U3FB-ROPS</v>
       </c>
       <c r="I526" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J526" t="str">
         <v>https://www.unimaticwatches.com</v>
@@ -22092,7 +22092,7 @@
         <v>Schallmauer Automatik</v>
       </c>
       <c r="I529" t="str">
-        <v>2024-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J529" t="str">
         <v>https://www.vandaag.de/en/</v>
@@ -22297,7 +22297,7 @@
         <v>Redentore Utopia II</v>
       </c>
       <c r="I534" t="str">
-        <v>2026-01-25</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J534" t="str">
         <v>https://www.venezianico.it</v>
@@ -23281,7 +23281,7 @@
         <v>Dunkirk Watch</v>
       </c>
       <c r="I558" t="str">
-        <v>2024-10-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J558" t="str">
         <v>https://www.williamwoodwatches.com</v>
@@ -23445,7 +23445,7 @@
         <v>Superman Titanium MoonTide CMM.11 Limited Edition</v>
       </c>
       <c r="I562" t="str">
-        <v>2024-10-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J562" t="str">
         <v>https://www.yema.com</v>
@@ -23650,7 +23650,7 @@
         <v/>
       </c>
       <c r="I567" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J567" t="str">
         <v>https://www.zenowatch.ch</v>
@@ -23691,7 +23691,7 @@
         <v>S6e Spitfire Escape</v>
       </c>
       <c r="I568" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J568" t="str">
         <v>https://zerowest.watch/</v>
@@ -23963,7 +23963,7 @@
         <v/>
       </c>
       <c r="I2" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J2" t="str">
         <v>https://www.5280watch.com</v>
@@ -24209,7 +24209,7 @@
         <v>Aquatico Automatic Dive Watch</v>
       </c>
       <c r="I8" t="str">
-        <v>2024-09-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J8" t="str">
         <v>https://www.aquaticowatches.com</v>
@@ -24291,7 +24291,7 @@
         <v>Caribe</v>
       </c>
       <c r="I10" t="str">
-        <v>2024-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J10" t="str">
         <v>https://ardiowatches.com/</v>
@@ -24496,7 +24496,7 @@
         <v>Terra Scout</v>
       </c>
       <c r="I15" t="str">
-        <v>2026-02-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J15" t="str">
         <v>https://astorandbanks.com</v>
@@ -24906,7 +24906,7 @@
         <v>Scarifour Automatic</v>
       </c>
       <c r="I25" t="str">
-        <v>2026-01-08</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J25" t="str">
         <v>https://benjaminjameswatches.com</v>
@@ -25029,7 +25029,7 @@
         <v/>
       </c>
       <c r="I28" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J28" t="str">
         <v>https://bernhardtwatch.com</v>
@@ -25152,7 +25152,7 @@
         <v>Odyssey MGP</v>
       </c>
       <c r="I31" t="str">
-        <v>2025-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J31" t="str">
         <v>https://www.boldrwatches.com</v>
@@ -25193,7 +25193,7 @@
         <v/>
       </c>
       <c r="I32" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J32" t="str">
         <v>https://www.borealiswatches.com</v>
@@ -25357,7 +25357,7 @@
         <v>Super Metric</v>
       </c>
       <c r="I36" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J36" t="str">
         <v>https://www.brew-watches.com</v>
@@ -25603,7 +25603,7 @@
         <v>Brooklyn Gent</v>
       </c>
       <c r="I42" t="str">
-        <v>2025-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J42" t="str">
         <v>https://carpenterwatches.com/</v>
@@ -25808,7 +25808,7 @@
         <v/>
       </c>
       <c r="I47" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J47" t="str">
         <v>https://www.cincinnatiwatchcompany.com</v>
@@ -25849,7 +25849,7 @@
         <v>Mechanic Ocean Mark II</v>
       </c>
       <c r="I48" t="str">
-        <v>2025-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J48" t="str">
         <v>https://www.crafterblue.com</v>
@@ -26177,7 +26177,7 @@
         <v>1975 Skin Diver</v>
       </c>
       <c r="I56" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J56" t="str">
         <v>https://www.danhenrywatches.com</v>
@@ -26505,7 +26505,7 @@
         <v>Westlake</v>
       </c>
       <c r="I64" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J64" t="str">
         <v>https://www.dufranewatches.com</v>
@@ -26956,7 +26956,7 @@
         <v>Seaplane Automatic</v>
       </c>
       <c r="I75" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J75" t="str">
         <v>https://www.farrandswit.com/</v>
@@ -27038,7 +27038,7 @@
         <v/>
       </c>
       <c r="I77" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J77" t="str">
         <v>https://www.feymantimekeepers.com</v>
@@ -27079,7 +27079,7 @@
         <v>FLX004</v>
       </c>
       <c r="I78" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J78" t="str">
         <v>https://www.fleuxwatches.com/</v>
@@ -27325,7 +27325,7 @@
         <v>Ocean Rover</v>
       </c>
       <c r="I84" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J84" t="str">
         <v>https://www.ginaultocean.com</v>
@@ -27366,7 +27366,7 @@
         <v/>
       </c>
       <c r="I85" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J85" t="str">
         <v>https://grandeur-usa.com/</v>
@@ -27612,7 +27612,7 @@
         <v/>
       </c>
       <c r="I91" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J91" t="str">
         <v>https://www.helmwatches.com</v>
@@ -27653,7 +27653,7 @@
         <v>Sky Racer</v>
       </c>
       <c r="I92" t="str">
-        <v>2024</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J92" t="str">
         <v>https://www.hemelwatches.com</v>
@@ -27694,7 +27694,7 @@
         <v>Bexley</v>
       </c>
       <c r="I93" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J93" t="str">
         <v>https://www.heritorwatches.com</v>
@@ -27940,7 +27940,7 @@
         <v/>
       </c>
       <c r="I99" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J99" t="str">
         <v>https://www.islanderwatches.com</v>
@@ -28555,7 +28555,7 @@
         <v>Astra</v>
       </c>
       <c r="I114" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J114" t="str">
         <v>https://www.lorierwatches.com</v>
@@ -28596,7 +28596,7 @@
         <v>M94 Bronze Date</v>
       </c>
       <c r="I115" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J115" t="str">
         <v>https://www.lum-tec.com</v>
@@ -29047,7 +29047,7 @@
         <v>Splash Eclipse</v>
       </c>
       <c r="I126" t="str">
-        <v>2024-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J126" t="str">
         <v>https://www.momentumwatch.com</v>
@@ -29088,7 +29088,7 @@
         <v>Triumph</v>
       </c>
       <c r="I127" t="str">
-        <v>2024-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J127" t="str">
         <v>https://www.montawatch.com</v>
@@ -29416,7 +29416,7 @@
         <v>Sector Deep</v>
       </c>
       <c r="I135" t="str">
-        <v>2024-12-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J135" t="str">
         <v>https://www.noduswatches.com</v>
@@ -29457,7 +29457,7 @@
         <v>Sentinel Collection</v>
       </c>
       <c r="I136" t="str">
-        <v>2024-12-19</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J136" t="str">
         <v>https://www.northernstarwatch.com/</v>
@@ -29662,7 +29662,7 @@
         <v>Core Diver</v>
       </c>
       <c r="I141" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J141" t="str">
         <v>https://www.oceancrawlerwatch.com</v>
@@ -29908,7 +29908,7 @@
         <v/>
       </c>
       <c r="I147" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J147" t="str">
         <v>https://www.orionwatches.com</v>
@@ -30113,7 +30113,7 @@
         <v>Jungle Field Automatic 38</v>
       </c>
       <c r="I152" t="str">
-        <v>2024-12-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J152" t="str">
         <v>https://www.praesidus.com</v>
@@ -30277,7 +30277,7 @@
         <v/>
       </c>
       <c r="I156" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J156" t="str">
         <v>https://www.ravenwatchco.com</v>
@@ -30318,7 +30318,7 @@
         <v>Crystal 2</v>
       </c>
       <c r="I157" t="str">
-        <v>2024-05-05</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J157" t="str">
         <v>https://www.reactorwatch.com</v>
@@ -30441,7 +30441,7 @@
         <v>Recon - C-47 Pathfinder (Full-Lume)</v>
       </c>
       <c r="I160" t="str">
-        <v>2024-11-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J160" t="str">
         <v>https://www.redwoodwatches.com</v>
@@ -32122,7 +32122,7 @@
         <v>Commuter</v>
       </c>
       <c r="I201" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J201" t="str">
         <v>https://www.traskawatch.com</v>
@@ -32245,7 +32245,7 @@
         <v>Torsk GMT 39</v>
       </c>
       <c r="I204" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J204" t="str">
         <v>https://www.tsaobaltimore.com</v>
@@ -32327,7 +32327,7 @@
         <v>C1 Ceremony Salmon</v>
       </c>
       <c r="I206" t="str">
-        <v>2024-12-19</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J206" t="str">
         <v>https://www.vaerwatches.com</v>
@@ -32614,7 +32614,7 @@
         <v>Duneshore Shallows</v>
       </c>
       <c r="I213" t="str">
-        <v>2025-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J213" t="str">
         <v>https://www.visitorwatchco.com/</v>
@@ -33024,7 +33024,7 @@
         <v/>
       </c>
       <c r="I223" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J223" t="str">
         <v>https://www.wolfpointwatches.com</v>
@@ -33065,7 +33065,7 @@
         <v>Enforcer</v>
       </c>
       <c r="I224" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J224" t="str">
         <v>https://www.xericdesigns.com</v>
@@ -33188,7 +33188,7 @@
         <v>Ultrathin</v>
       </c>
       <c r="I227" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J227" t="str">
         <v>https://www.zeloswatch.com</v>
@@ -33337,7 +33337,7 @@
         <v>Horizon Voyager</v>
       </c>
       <c r="I3" t="str">
-        <v>2024-12-19</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J3" t="str">
         <v>https://aethelsohnwatch.com/</v>
@@ -33378,7 +33378,7 @@
         <v>Volcano</v>
       </c>
       <c r="I4" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J4" t="str">
         <v>https://agelocer.com</v>
@@ -33419,7 +33419,7 @@
         <v>Kakori 8 Down- Centenary Edition</v>
       </c>
       <c r="I5" t="str">
-        <v>2026-03-27</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J5" t="str">
         <v>https://ajwa.in/</v>
@@ -33501,7 +33501,7 @@
         <v>Voyager Worldtimer GMT</v>
       </c>
       <c r="I7" t="str">
-        <v>2024-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J7" t="str">
         <v>https://alcadus.com/</v>
@@ -33665,7 +33665,7 @@
         <v>Inflection</v>
       </c>
       <c r="I11" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J11" t="str">
         <v>https://www.atelierwen.com</v>
@@ -33788,7 +33788,7 @@
         <v/>
       </c>
       <c r="I14" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J14" t="str">
         <v>https://awakewatches.com.au</v>
@@ -33911,7 +33911,7 @@
         <v/>
       </c>
       <c r="I17" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J17" t="str">
         <v>https://bangalorewatch.com</v>
@@ -34116,7 +34116,7 @@
         <v>Voyager Chronograph</v>
       </c>
       <c r="I22" t="str">
-        <v>2024-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J22" t="str">
         <v>https://www.boderry.com</v>
@@ -34362,7 +34362,7 @@
         <v/>
       </c>
       <c r="I28" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J28" t="str">
         <v>https://www.cigadesign.com</v>
@@ -34567,7 +34567,7 @@
         <v>DW-D3</v>
       </c>
       <c r="I33" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J33" t="str">
         <v>https://www.duzuwatches.com/</v>
@@ -34608,7 +34608,7 @@
         <v/>
       </c>
       <c r="I34" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J34" t="str">
         <v>https://www.earthenco.com</v>
@@ -35059,7 +35059,7 @@
         <v>Broadway 40</v>
       </c>
       <c r="I45" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J45" t="str">
         <v>https://www.havaantuvali.com/</v>
@@ -35264,7 +35264,7 @@
         <v>Pilbara Rock Dive Watch - Second Release</v>
       </c>
       <c r="I50" t="str">
-        <v>2024-12-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J50" t="str">
         <v>https://houtmanwatch.com/</v>
@@ -35674,7 +35674,7 @@
         <v/>
       </c>
       <c r="I60" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J60" t="str">
         <v>https://kiwametokyo.com/en/collections/watches</v>
@@ -35756,7 +35756,7 @@
         <v/>
       </c>
       <c r="I62" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J62" t="str">
         <v>https://www.kuoe-en.com/</v>
@@ -35838,7 +35838,7 @@
         <v>Kronosprinter</v>
       </c>
       <c r="I64" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J64" t="str">
         <v>https://us.limawatch.com/</v>
@@ -35920,7 +35920,7 @@
         <v>Moana</v>
       </c>
       <c r="I66" t="str">
-        <v>2024-05-10</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J66" t="str">
         <v>https://www.magrette.com</v>
@@ -36289,7 +36289,7 @@
         <v/>
       </c>
       <c r="I75" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J75" t="str">
         <v>https://www.melbournewatchco.com</v>
@@ -36412,7 +36412,7 @@
         <v>37.09 Bluefin</v>
       </c>
       <c r="I78" t="str">
-        <v>2024-12-31</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J78" t="str">
         <v>https://www.ming.watch</v>
@@ -36658,7 +36658,7 @@
         <v>BALEINE – 202</v>
       </c>
       <c r="I84" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J84" t="str">
         <v>https://www.nezumistudios.com</v>
@@ -36699,7 +36699,7 @@
         <v>Himalayan Project</v>
       </c>
       <c r="I85" t="str">
-        <v>2024-04-15</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J85" t="str">
         <v>https://www.oceantoorbit.com/</v>
@@ -36904,7 +36904,7 @@
         <v>Storm Corsair</v>
       </c>
       <c r="I90" t="str">
-        <v>2024-04-06</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J90" t="str">
         <v>https://www.phoiboswatch.com</v>
@@ -37396,7 +37396,7 @@
         <v>The Fusion</v>
       </c>
       <c r="I102" t="str">
-        <v>2024-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J102" t="str">
         <v>https://www.secondhour.com.au</v>
@@ -37888,7 +37888,7 @@
         <v>1918 Trench &amp; Medic</v>
       </c>
       <c r="I114" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J114" t="str">
         <v>https://www.vario.sg</v>
@@ -37970,7 +37970,7 @@
         <v/>
       </c>
       <c r="I116" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J116" t="str">
         <v>https://wancherwatch.com/</v>
@@ -38339,7 +38339,7 @@
         <v/>
       </c>
       <c r="I125" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J125" t="str">
         <v>https://www.zeroo.jp</v>
@@ -40333,7 +40333,7 @@
         <v>Fieldtimer</v>
       </c>
       <c r="I47" t="str">
-        <v>2025-11-25</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J47" t="str">
         <v>https://campwatches.com/</v>
@@ -41071,7 +41071,7 @@
         <v>Gatekeeper</v>
       </c>
       <c r="I65" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J65" t="str">
         <v>https://decima-watches.com/</v>
@@ -41317,7 +41317,7 @@
         <v>DRZ 07 Universo</v>
       </c>
       <c r="I71" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J71" t="str">
         <v>https://direnzowatches.com/</v>
@@ -41809,7 +41809,7 @@
         <v/>
       </c>
       <c r="I83" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J83" t="str">
         <v>https://englemaan.com</v>
@@ -41850,7 +41850,7 @@
         <v>Twenty-Four</v>
       </c>
       <c r="I84" t="str">
-        <v>2024-12-19</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J84" t="str">
         <v>https://erebuswatches.com/</v>
@@ -42465,7 +42465,7 @@
         <v>March 5</v>
       </c>
       <c r="I99" t="str">
-        <v>2025-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J99" t="str">
         <v>https://watchesgalo.com/</v>
@@ -42957,7 +42957,7 @@
         <v/>
       </c>
       <c r="I111" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J111" t="str">
         <v>https://halcyonwatch.com/</v>
@@ -43039,7 +43039,7 @@
         <v/>
       </c>
       <c r="I113" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J113" t="str">
         <v>https://havenwatchco.com/</v>
@@ -43367,7 +43367,7 @@
         <v>Racing 40</v>
       </c>
       <c r="I121" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J121" t="str">
         <v>https://hoffmanwatches.com/</v>
@@ -43613,7 +43613,7 @@
         <v>Aquatique GMT</v>
       </c>
       <c r="I127" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J127" t="str">
         <v>https://hultwatches.com/</v>
@@ -43982,7 +43982,7 @@
         <v>IXDAO Pilot Series</v>
       </c>
       <c r="I136" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J136" t="str">
         <v>https://ixdaowatches.com/</v>
@@ -44597,7 +44597,7 @@
         <v>Chiming Watch 2.0</v>
       </c>
       <c r="I151" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J151" t="str">
         <v>https://luckyharveywatch.com/</v>
@@ -44925,7 +44925,7 @@
         <v>Odyssey: Baja</v>
       </c>
       <c r="I159" t="str">
-        <v>2026-01-26</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J159" t="str">
         <v>https://www.marininstruments.com/</v>
@@ -44966,7 +44966,7 @@
         <v>M 6</v>
       </c>
       <c r="I160" t="str">
-        <v>2024-12-15</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J160" t="str">
         <v>https://marktimewatches.com/</v>
@@ -45335,7 +45335,7 @@
         <v>Milifortic S103</v>
       </c>
       <c r="I169" t="str">
-        <v>2024-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J169" t="str">
         <v>https://miliforticwatch.com/</v>
@@ -45540,7 +45540,7 @@
         <v>MB3 TRINOVA</v>
       </c>
       <c r="I174" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J174" t="str">
         <v>https://monbrey.com/</v>
@@ -45909,7 +45909,7 @@
         <v>Vespera GMT</v>
       </c>
       <c r="I183" t="str">
-        <v>2026-03-09</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J183" t="str">
         <v>https://nadirwatches.com/</v>
@@ -46032,7 +46032,7 @@
         <v>SHIRAHAMA 2</v>
       </c>
       <c r="I186" t="str">
-        <v>2024-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J186" t="str">
         <v>https://www.namicawatches.com/</v>
@@ -46524,7 +46524,7 @@
         <v>LUNØR</v>
       </c>
       <c r="I198" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J198" t="str">
         <v>https://nordicmarineinstruments.com/</v>
@@ -47508,7 +47508,7 @@
         <v>Onward Future Field Watch</v>
       </c>
       <c r="I222" t="str">
-        <v>2024-12-31</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J222" t="str">
         <v>https://prevailwatches.com/</v>
@@ -47836,7 +47836,7 @@
         <v>Terra 38 Casablanca</v>
       </c>
       <c r="I230" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J230" t="str">
         <v>https://www.revelot.com/</v>
@@ -48779,7 +48779,7 @@
         <v>VisiLume GMT</v>
       </c>
       <c r="I253" t="str">
-        <v>2024-12-19</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J253" t="str">
         <v>https://sheffieldwatches.com/</v>
@@ -50050,7 +50050,7 @@
         <v>Daytripper Season Two</v>
       </c>
       <c r="I284" t="str">
-        <v>2024-12-19</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J284" t="str">
         <v>https://www.traffordwatchco.com/</v>
@@ -50255,7 +50255,7 @@
         <v>Adamas Aster</v>
       </c>
       <c r="I289" t="str">
-        <v>2026-01-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J289" t="str">
         <v>https://uglywatchco.com/</v>
@@ -50501,7 +50501,7 @@
         <v>Northstar N-8 'Full Lume'</v>
       </c>
       <c r="I295" t="str">
-        <v/>
+        <v>2026-04-04</v>
       </c>
       <c r="J295" t="str">
         <v>https://ventuswatches.com/</v>
@@ -50829,7 +50829,7 @@
         <v>WIC006 GMT</v>
       </c>
       <c r="I303" t="str">
-        <v>2024-10-01</v>
+        <v>2026-04-04</v>
       </c>
       <c r="J303" t="str">
         <v>https://www.wickedwatch.ch/</v>
@@ -51569,7 +51569,7 @@
         <v>Last Updated</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-04-02</v>
+        <v>2026-04-04</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
feat: re-enrich all four regions — prices, models, founded years, notes
</commit_message>
<xml_diff>
--- a/watch-microbrand-database.xlsx
+++ b/watch-microbrand-database.xlsx
@@ -590,7 +590,7 @@
         <v>United Kingdom</v>
       </c>
       <c r="C5" t="str">
-        <v/>
+        <v>Tetbury</v>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -713,7 +713,7 @@
         <v>Switzerland</v>
       </c>
       <c r="C8" t="str">
-        <v/>
+        <v>Geneva</v>
       </c>
       <c r="D8">
         <v>1894</v>
@@ -836,7 +836,7 @@
         <v>Switzerland</v>
       </c>
       <c r="C11" t="str">
-        <v>Les Brenets</v>
+        <v>Saignelégier</v>
       </c>
       <c r="D11">
         <v>1942</v>
@@ -851,10 +851,10 @@
         <v>Active</v>
       </c>
       <c r="H11" t="str">
-        <v/>
+        <v>Renaissance Squelette Cobweb</v>
       </c>
       <c r="I11" t="str">
-        <v/>
+        <v>2019-01-01</v>
       </c>
       <c r="J11" t="str">
         <v>https://www.aerowatch.ch</v>
@@ -997,7 +997,7 @@
         <v>AIRIN</v>
       </c>
       <c r="B15" t="str">
-        <v>France</v>
+        <v>Switzerland</v>
       </c>
       <c r="C15" t="str">
         <v/>
@@ -1656,7 +1656,7 @@
         <v>Germany</v>
       </c>
       <c r="C31" t="str">
-        <v/>
+        <v>Hamburg</v>
       </c>
       <c r="D31">
         <v>1960</v>
@@ -1721,7 +1721,7 @@
         <v>https://aquastar.ch/</v>
       </c>
       <c r="K32" t="str">
-        <v/>
+        <v>aquastarwatches</v>
       </c>
       <c r="L32" t="str">
         <v>MBWDB</v>
@@ -1738,7 +1738,7 @@
         <v>France</v>
       </c>
       <c r="C33" t="str">
-        <v>Paris</v>
+        <v>Grenoble</v>
       </c>
       <c r="D33" t="str">
         <v/>
@@ -1861,7 +1861,7 @@
         <v>Germany</v>
       </c>
       <c r="C36" t="str">
-        <v/>
+        <v>Pforzheim</v>
       </c>
       <c r="D36">
         <v>1924</v>
@@ -1943,7 +1943,7 @@
         <v>Switzerland</v>
       </c>
       <c r="C38" t="str">
-        <v/>
+        <v>Tramelan</v>
       </c>
       <c r="D38">
         <v>1875</v>
@@ -1961,7 +1961,7 @@
         <v>M02 Special Edition Toni Art</v>
       </c>
       <c r="I38" t="str">
-        <v/>
+        <v>2024-11-01</v>
       </c>
       <c r="J38" t="str">
         <v>https://www.armandnicolet.com</v>
@@ -2025,16 +2025,16 @@
         <v>Germany</v>
       </c>
       <c r="C40" t="str">
-        <v>Berlin</v>
+        <v>Rathenow</v>
       </c>
       <c r="D40" t="str">
         <v/>
       </c>
-      <c r="E40" t="str">
-        <v/>
-      </c>
-      <c r="F40" t="str">
-        <v/>
+      <c r="E40">
+        <v>39</v>
+      </c>
+      <c r="F40">
+        <v>10700</v>
       </c>
       <c r="G40" t="str">
         <v>Active</v>
@@ -2268,7 +2268,7 @@
         <v>Augmé</v>
       </c>
       <c r="B46" t="str">
-        <v>France</v>
+        <v>Denmark</v>
       </c>
       <c r="C46" t="str">
         <v>Paris</v>
@@ -2286,7 +2286,7 @@
         <v>Active</v>
       </c>
       <c r="H46" t="str">
-        <v/>
+        <v>Serenity Petite</v>
       </c>
       <c r="I46" t="str">
         <v/>
@@ -2295,7 +2295,7 @@
         <v>https://augustberg.com/</v>
       </c>
       <c r="K46" t="str">
-        <v/>
+        <v>augustbergofficial</v>
       </c>
       <c r="L46" t="str">
         <v>existing-db</v>
@@ -2645,11 +2645,11 @@
       <c r="D55">
         <v>1903</v>
       </c>
-      <c r="E55" t="str">
-        <v/>
-      </c>
-      <c r="F55" t="str">
-        <v/>
+      <c r="E55">
+        <v>425</v>
+      </c>
+      <c r="F55">
+        <v>900</v>
       </c>
       <c r="G55" t="str">
         <v>Active</v>
@@ -2658,13 +2658,13 @@
         <v>Holland Automatic BL-3150-03</v>
       </c>
       <c r="I55" t="str">
-        <v/>
+        <v>2024-12-01</v>
       </c>
       <c r="J55" t="str">
         <v>https://www.ballast1903.com/</v>
       </c>
       <c r="K55" t="str">
-        <v/>
+        <v>ballast1903</v>
       </c>
       <c r="L55" t="str">
         <v>MBWDB</v>
@@ -2845,7 +2845,7 @@
         <v>United Kingdom</v>
       </c>
       <c r="C60" t="str">
-        <v/>
+        <v>London</v>
       </c>
       <c r="D60">
         <v>2002</v>
@@ -2886,16 +2886,16 @@
         <v>Netherlands</v>
       </c>
       <c r="C61" t="str">
-        <v>Amsterdam</v>
+        <v>Tilburg</v>
       </c>
       <c r="D61" t="str">
         <v/>
       </c>
-      <c r="E61" t="str">
-        <v/>
-      </c>
-      <c r="F61" t="str">
-        <v/>
+      <c r="E61">
+        <v>26</v>
+      </c>
+      <c r="F61">
+        <v>710</v>
       </c>
       <c r="G61" t="str">
         <v>Active</v>
@@ -2904,13 +2904,13 @@
         <v>Batavi Geograaf</v>
       </c>
       <c r="I61" t="str">
-        <v/>
+        <v>2025-01-01</v>
       </c>
       <c r="J61" t="str">
         <v>https://www.batavi-watches.com/</v>
       </c>
       <c r="K61" t="str">
-        <v/>
+        <v>batavi_watches</v>
       </c>
       <c r="L61" t="str">
         <v>MBWDB</v>
@@ -2927,7 +2927,7 @@
         <v>Hong Kong</v>
       </c>
       <c r="C62" t="str">
-        <v>Kwun Tong</v>
+        <v>Hong Kong</v>
       </c>
       <c r="D62" t="str">
         <v/>
@@ -3091,7 +3091,7 @@
         <v>Italy</v>
       </c>
       <c r="C66" t="str">
-        <v>Roma</v>
+        <v>Rome</v>
       </c>
       <c r="D66">
         <v>1882</v>
@@ -3419,7 +3419,7 @@
         <v>Slovakia</v>
       </c>
       <c r="C74" t="str">
-        <v/>
+        <v>Banská Bystrica</v>
       </c>
       <c r="D74">
         <v>2010</v>
@@ -3601,7 +3601,7 @@
         <v>MNGRA</v>
       </c>
       <c r="I78" t="str">
-        <v/>
+        <v>2024-12-01</v>
       </c>
       <c r="J78" t="str">
         <v>https://bnd-watches.com/?lang=en</v>
@@ -3665,7 +3665,7 @@
         <v>Switzerland</v>
       </c>
       <c r="C80" t="str">
-        <v/>
+        <v>Neuchâtel</v>
       </c>
       <c r="D80" t="str">
         <v/>
@@ -3788,7 +3788,7 @@
         <v>Germany</v>
       </c>
       <c r="C83" t="str">
-        <v/>
+        <v>Königstein</v>
       </c>
       <c r="D83">
         <v>1986</v>
@@ -4154,7 +4154,7 @@
         <v>Briston</v>
       </c>
       <c r="B92" t="str">
-        <v>France</v>
+        <v>United Kingdom</v>
       </c>
       <c r="C92" t="str">
         <v>Paris</v>
@@ -4198,7 +4198,7 @@
         <v>France</v>
       </c>
       <c r="C93" t="str">
-        <v/>
+        <v>Paris</v>
       </c>
       <c r="D93">
         <v>2005</v>
@@ -4321,7 +4321,7 @@
         <v>Norway</v>
       </c>
       <c r="C96" t="str">
-        <v/>
+        <v>Oslo</v>
       </c>
       <c r="D96" t="str">
         <v/>
@@ -4690,16 +4690,16 @@
         <v>Switzerland</v>
       </c>
       <c r="C105" t="str">
-        <v>Les Breuleux</v>
+        <v>Uznach</v>
       </c>
       <c r="D105">
         <v>1858</v>
       </c>
-      <c r="E105" t="str">
-        <v/>
-      </c>
-      <c r="F105" t="str">
-        <v/>
+      <c r="E105">
+        <v>400</v>
+      </c>
+      <c r="F105">
+        <v>1200</v>
       </c>
       <c r="G105" t="str">
         <v>Active</v>
@@ -4728,7 +4728,7 @@
         <v>Celadon (Maison Celadon Watches)</v>
       </c>
       <c r="B106" t="str">
-        <v>France</v>
+        <v>China</v>
       </c>
       <c r="C106" t="str">
         <v/>
@@ -5228,11 +5228,11 @@
       <c r="D118">
         <v>2014</v>
       </c>
-      <c r="E118" t="str">
-        <v/>
-      </c>
-      <c r="F118" t="str">
-        <v/>
+      <c r="E118">
+        <v>499</v>
+      </c>
+      <c r="F118">
+        <v>2388</v>
       </c>
       <c r="G118" t="str">
         <v>Active</v>
@@ -5241,13 +5241,13 @@
         <v>Airspeed</v>
       </c>
       <c r="I118" t="str">
-        <v/>
+        <v>2021-01-01</v>
       </c>
       <c r="J118" t="str">
         <v>https://www.cjrwatches.com</v>
       </c>
       <c r="K118" t="str">
-        <v/>
+        <v>cjrwatches</v>
       </c>
       <c r="L118" t="str">
         <v>MBWDB</v>
@@ -5305,7 +5305,7 @@
         <v>Denmark</v>
       </c>
       <c r="C120" t="str">
-        <v>Copenhagen</v>
+        <v>St Andrews</v>
       </c>
       <c r="D120" t="str">
         <v/>
@@ -5540,7 +5540,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M125" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>UK-based military watch brand specializing in diver watches and vintage military-inspired timepieces. Product range includes Royal Navy style divers watches, WW2 pattern German Luftwaffe replicas, and modern tactical military watches with water resistance up to 300m.</v>
       </c>
     </row>
     <row r="126">
@@ -5592,7 +5592,7 @@
         <v>Switzerland</v>
       </c>
       <c r="C127" t="str">
-        <v>Zurich</v>
+        <v>Geneva</v>
       </c>
       <c r="D127">
         <v>2010</v>
@@ -6852,7 +6852,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M157" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>Italian watch brand featuring diver watches and neo-vintage timepieces. Collections include models like Patriota, Amalfi, and Fano with movements including automatic and mecha-quartz chronographs. Currently selling 110 watch models in stock.</v>
       </c>
     </row>
     <row r="158">
@@ -6863,7 +6863,7 @@
         <v>Switzerland</v>
       </c>
       <c r="C158" t="str">
-        <v>Neuchâtel</v>
+        <v>Cormondrèche</v>
       </c>
       <c r="D158">
         <v>2016</v>
@@ -7032,11 +7032,11 @@
       <c r="D162">
         <v>2019</v>
       </c>
-      <c r="E162" t="str">
-        <v/>
-      </c>
-      <c r="F162" t="str">
-        <v/>
+      <c r="E162">
+        <v>528</v>
+      </c>
+      <c r="F162">
+        <v>556</v>
       </c>
       <c r="G162" t="str">
         <v>Active</v>
@@ -7045,7 +7045,7 @@
         <v>DV-02</v>
       </c>
       <c r="I162" t="str">
-        <v/>
+        <v>2025-01-01</v>
       </c>
       <c r="J162" t="str">
         <v>https://draytonwatches.com/</v>
@@ -7191,7 +7191,7 @@
         <v>United Kingdom</v>
       </c>
       <c r="C166" t="str">
-        <v/>
+        <v>Bolton</v>
       </c>
       <c r="D166">
         <v>1920</v>
@@ -7232,7 +7232,7 @@
         <v>Germany</v>
       </c>
       <c r="C167" t="str">
-        <v/>
+        <v>Hamburg</v>
       </c>
       <c r="D167">
         <v>2007</v>
@@ -7273,7 +7273,7 @@
         <v>Switzerland</v>
       </c>
       <c r="C168" t="str">
-        <v/>
+        <v>Lugano</v>
       </c>
       <c r="D168">
         <v>2011</v>
@@ -7281,8 +7281,8 @@
       <c r="E168">
         <v>1400</v>
       </c>
-      <c r="F168" t="str">
-        <v/>
+      <c r="F168">
+        <v>1347</v>
       </c>
       <c r="G168" t="str">
         <v>Active</v>
@@ -7291,7 +7291,7 @@
         <v>A1</v>
       </c>
       <c r="I168" t="str">
-        <v/>
+        <v>2026-01-01</v>
       </c>
       <c r="J168" t="str">
         <v>https://www.dwiss.com</v>
@@ -7314,7 +7314,7 @@
         <v>United Kingdom</v>
       </c>
       <c r="C169" t="str">
-        <v/>
+        <v>London</v>
       </c>
       <c r="D169">
         <v>2013</v>
@@ -7396,7 +7396,7 @@
         <v>Italy</v>
       </c>
       <c r="C171" t="str">
-        <v>Milan, Italy</v>
+        <v>Milano</v>
       </c>
       <c r="D171">
         <v>2019</v>
@@ -7434,7 +7434,7 @@
         <v>Edmond</v>
       </c>
       <c r="B172" t="str">
-        <v>Sweden</v>
+        <v>Switzerland</v>
       </c>
       <c r="C172" t="str">
         <v/>
@@ -7724,7 +7724,7 @@
         <v>United Kingdom</v>
       </c>
       <c r="C179" t="str">
-        <v/>
+        <v>Kendal</v>
       </c>
       <c r="D179">
         <v>2012</v>
@@ -7847,7 +7847,7 @@
         <v>Switzerland</v>
       </c>
       <c r="C182" t="str">
-        <v/>
+        <v>La Chaux de Fonds</v>
       </c>
       <c r="D182">
         <v>1948</v>
@@ -7871,7 +7871,7 @@
         <v>http://www.enicar.com/</v>
       </c>
       <c r="K182" t="str">
-        <v/>
+        <v>enicarswiss</v>
       </c>
       <c r="L182" t="str">
         <v>MBWDB</v>
@@ -8000,7 +8000,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M185" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>German watchmaker Roland Kemmner, former Fricker employee, builds custom Marine-style watches inspired by WW2 Kriegsmarine designs. Offers affordable alternatives featuring Swiss Unitas movements and 316L steel cases, sold through eBay shop Erkahund with direct commission options.</v>
       </c>
     </row>
     <row r="186">
@@ -8180,11 +8180,11 @@
       <c r="D190" t="str">
         <v/>
       </c>
-      <c r="E190" t="str">
-        <v/>
-      </c>
-      <c r="F190" t="str">
-        <v/>
+      <c r="E190">
+        <v>1057</v>
+      </c>
+      <c r="F190">
+        <v>1271</v>
       </c>
       <c r="G190" t="str">
         <v>Active</v>
@@ -8544,7 +8544,7 @@
         <v>United States</v>
       </c>
       <c r="C199" t="str">
-        <v>Indiana</v>
+        <v>Indianapolis</v>
       </c>
       <c r="D199" t="str">
         <v/>
@@ -8603,7 +8603,7 @@
         <v>FLORIJN</v>
       </c>
       <c r="I200" t="str">
-        <v/>
+        <v>2017-05-01</v>
       </c>
       <c r="J200" t="str">
         <v>https://www.blessthisstuff.com/stuff/wear/watches/florijn-watch/</v>
@@ -8913,7 +8913,7 @@
         <v>United Kingdom</v>
       </c>
       <c r="C208" t="str">
-        <v>Norwich</v>
+        <v>Norfolk</v>
       </c>
       <c r="D208" t="str">
         <v/>
@@ -9036,16 +9036,16 @@
         <v>Poland</v>
       </c>
       <c r="C211" t="str">
-        <v/>
+        <v>Szczecin</v>
       </c>
       <c r="D211" t="str">
         <v/>
       </c>
-      <c r="E211" t="str">
-        <v/>
-      </c>
-      <c r="F211" t="str">
-        <v/>
+      <c r="E211">
+        <v>700</v>
+      </c>
+      <c r="F211">
+        <v>1000</v>
       </c>
       <c r="G211" t="str">
         <v>Active</v>
@@ -9115,28 +9115,28 @@
         <v>Giorgio Martino</v>
       </c>
       <c r="B213" t="str">
-        <v>Italy</v>
+        <v>United Kingdom</v>
       </c>
       <c r="C213" t="str">
-        <v/>
-      </c>
-      <c r="D213" t="str">
-        <v/>
-      </c>
-      <c r="E213" t="str">
-        <v/>
-      </c>
-      <c r="F213" t="str">
-        <v/>
+        <v>London</v>
+      </c>
+      <c r="D213">
+        <v>2020</v>
+      </c>
+      <c r="E213">
+        <v>52</v>
+      </c>
+      <c r="F213">
+        <v>107</v>
       </c>
       <c r="G213" t="str">
         <v>Active</v>
       </c>
       <c r="H213" t="str">
-        <v/>
+        <v>VEROSTY GX 650</v>
       </c>
       <c r="I213" t="str">
-        <v/>
+        <v>2025-01-01</v>
       </c>
       <c r="J213" t="str">
         <v>https://giorgiomartino.club/</v>
@@ -9530,29 +9530,29 @@
       <c r="C223" t="str">
         <v>Frankfurt am Main</v>
       </c>
-      <c r="D223" t="str">
-        <v/>
-      </c>
-      <c r="E223" t="str">
-        <v/>
-      </c>
-      <c r="F223" t="str">
-        <v/>
+      <c r="D223">
+        <v>1865</v>
+      </c>
+      <c r="E223">
+        <v>1800</v>
+      </c>
+      <c r="F223">
+        <v>2500</v>
       </c>
       <c r="G223" t="str">
         <v>Active</v>
       </c>
       <c r="H223" t="str">
-        <v/>
+        <v>Deepwave Whitewater</v>
       </c>
       <c r="I223" t="str">
-        <v/>
+        <v>2024-09-03</v>
       </c>
       <c r="J223" t="str">
         <v>https://www.guinand-uhren.de/home-en.html</v>
       </c>
       <c r="K223" t="str">
-        <v/>
+        <v>guinandwatches</v>
       </c>
       <c r="L223" t="str">
         <v>MBWDB</v>
@@ -9628,7 +9628,7 @@
         <v>NAVI S</v>
       </c>
       <c r="I225" t="str">
-        <v/>
+        <v>2025-01-01</v>
       </c>
       <c r="J225" t="str">
         <v>https://gyavius.com/about</v>
@@ -9651,7 +9651,7 @@
         <v>Switzerland</v>
       </c>
       <c r="C226" t="str">
-        <v/>
+        <v>Schaffhausen</v>
       </c>
       <c r="D226">
         <v>1828</v>
@@ -9856,7 +9856,7 @@
         <v>Sweden</v>
       </c>
       <c r="C231" t="str">
-        <v>Svängsta</v>
+        <v>Sollentuna</v>
       </c>
       <c r="D231">
         <v>1887</v>
@@ -9938,7 +9938,7 @@
         <v>Germany</v>
       </c>
       <c r="C233" t="str">
-        <v/>
+        <v>Schonachbach</v>
       </c>
       <c r="D233">
         <v>1882</v>
@@ -10315,8 +10315,8 @@
       <c r="E242">
         <v>360</v>
       </c>
-      <c r="F242" t="str">
-        <v/>
+      <c r="F242">
+        <v>550</v>
       </c>
       <c r="G242" t="str">
         <v>Active</v>
@@ -10348,7 +10348,7 @@
         <v>Netherlands</v>
       </c>
       <c r="C243" t="str">
-        <v/>
+        <v>Delft</v>
       </c>
       <c r="D243">
         <v>2016</v>
@@ -10430,7 +10430,7 @@
         <v>Netherlands</v>
       </c>
       <c r="C245" t="str">
-        <v>Heerde, Netherlands</v>
+        <v>Heerde</v>
       </c>
       <c r="D245">
         <v>2014</v>
@@ -10473,23 +10473,23 @@
       <c r="C246" t="str">
         <v>Besançon</v>
       </c>
-      <c r="D246" t="str">
-        <v/>
-      </c>
-      <c r="E246" t="str">
-        <v/>
-      </c>
-      <c r="F246" t="str">
-        <v/>
+      <c r="D246">
+        <v>1964</v>
+      </c>
+      <c r="E246">
+        <v>699</v>
+      </c>
+      <c r="F246">
+        <v>1090</v>
       </c>
       <c r="G246" t="str">
         <v>Active</v>
       </c>
       <c r="H246" t="str">
-        <v/>
+        <v>HD6.1 Chronographe</v>
       </c>
       <c r="I246" t="str">
-        <v/>
+        <v>2024-01-01</v>
       </c>
       <c r="J246" t="str">
         <v>https://www.humbert-droz.fr/en/</v>
@@ -10758,7 +10758,7 @@
         <v>Germany</v>
       </c>
       <c r="C253" t="str">
-        <v/>
+        <v>Hamburg</v>
       </c>
       <c r="D253">
         <v>2014</v>
@@ -10796,7 +10796,7 @@
         <v>Isotope</v>
       </c>
       <c r="B254" t="str">
-        <v>England</v>
+        <v>United Kingdom</v>
       </c>
       <c r="C254" t="str">
         <v>Henfield</v>
@@ -10858,7 +10858,7 @@
         <v>New Series</v>
       </c>
       <c r="I255" t="str">
-        <v/>
+        <v>2024-10-01</v>
       </c>
       <c r="J255" t="str">
         <v>https://www.jacobjensen.com</v>
@@ -11009,26 +11009,26 @@
       <c r="D259" t="str">
         <v/>
       </c>
-      <c r="E259" t="str">
-        <v/>
-      </c>
-      <c r="F259" t="str">
-        <v/>
+      <c r="E259">
+        <v>230</v>
+      </c>
+      <c r="F259">
+        <v>390</v>
       </c>
       <c r="G259" t="str">
         <v>Active</v>
       </c>
       <c r="H259" t="str">
-        <v/>
+        <v>Rally Automatic</v>
       </c>
       <c r="I259" t="str">
-        <v/>
+        <v>2024-12-19</v>
       </c>
       <c r="J259" t="str">
         <v>https://mccabewatches.com/</v>
       </c>
       <c r="K259" t="str">
-        <v/>
+        <v>mccabewatches</v>
       </c>
       <c r="L259" t="str">
         <v>MBWDB</v>
@@ -11045,7 +11045,7 @@
         <v>Switzerland</v>
       </c>
       <c r="C260" t="str">
-        <v/>
+        <v>Grenchen</v>
       </c>
       <c r="D260">
         <v>1992</v>
@@ -11129,14 +11129,14 @@
       <c r="C262" t="str">
         <v/>
       </c>
-      <c r="D262" t="str">
-        <v/>
-      </c>
-      <c r="E262" t="str">
-        <v/>
-      </c>
-      <c r="F262" t="str">
-        <v/>
+      <c r="D262">
+        <v>2012</v>
+      </c>
+      <c r="E262">
+        <v>195</v>
+      </c>
+      <c r="F262">
+        <v>495</v>
       </c>
       <c r="G262" t="str">
         <v>Active</v>
@@ -11151,7 +11151,7 @@
         <v>https://www.jorggrey.com</v>
       </c>
       <c r="K262" t="str">
-        <v/>
+        <v>jorggreyofficial</v>
       </c>
       <c r="L262" t="str">
         <v>MBWDB</v>
@@ -11211,8 +11211,8 @@
       <c r="C264" t="str">
         <v>Reykjavik</v>
       </c>
-      <c r="D264" t="str">
-        <v/>
+      <c r="D264">
+        <v>2004</v>
       </c>
       <c r="E264" t="str">
         <v/>
@@ -11224,7 +11224,7 @@
         <v>Active</v>
       </c>
       <c r="H264" t="str">
-        <v/>
+        <v>SIF Protector Special Edition</v>
       </c>
       <c r="I264" t="str">
         <v>2026-04-04</v>
@@ -11233,7 +11233,7 @@
         <v>https://www.jswatch.com</v>
       </c>
       <c r="K264" t="str">
-        <v/>
+        <v>jswatch</v>
       </c>
       <c r="L264" t="str">
         <v>MBWDB</v>
@@ -11291,7 +11291,7 @@
         <v>Germany</v>
       </c>
       <c r="C266" t="str">
-        <v/>
+        <v>Schramberg</v>
       </c>
       <c r="D266">
         <v>1897</v>
@@ -11370,7 +11370,7 @@
         <v>K.Grun &amp; Sohne</v>
       </c>
       <c r="B268" t="str">
-        <v>Switzerland</v>
+        <v>United Kingdom</v>
       </c>
       <c r="C268" t="str">
         <v>Surrey</v>
@@ -11501,11 +11501,11 @@
       <c r="D271" t="str">
         <v/>
       </c>
-      <c r="E271" t="str">
-        <v/>
-      </c>
-      <c r="F271" t="str">
-        <v/>
+      <c r="E271">
+        <v>399</v>
+      </c>
+      <c r="F271">
+        <v>399</v>
       </c>
       <c r="G271" t="str">
         <v>Active</v>
@@ -11514,13 +11514,13 @@
         <v>Baltic Shield</v>
       </c>
       <c r="I271" t="str">
-        <v/>
+        <v>2022-12-31</v>
       </c>
       <c r="J271" t="str">
         <v>https://www.karlskronawatch.com/</v>
       </c>
       <c r="K271" t="str">
-        <v/>
+        <v>karlskronawatch</v>
       </c>
       <c r="L271" t="str">
         <v>MBWDB</v>
@@ -11575,7 +11575,7 @@
         <v>Kazimon</v>
       </c>
       <c r="B273" t="str">
-        <v>Germany</v>
+        <v>Switzerland</v>
       </c>
       <c r="C273" t="str">
         <v>Steinhausen</v>
@@ -11952,8 +11952,8 @@
       <c r="D282">
         <v>2020</v>
       </c>
-      <c r="E282" t="str">
-        <v/>
+      <c r="E282">
+        <v>2500</v>
       </c>
       <c r="F282">
         <v>152352</v>
@@ -11971,7 +11971,7 @@
         <v>https://www.krossstudio.com</v>
       </c>
       <c r="K282" t="str">
-        <v/>
+        <v>kross_studio</v>
       </c>
       <c r="L282" t="str">
         <v>existing-db</v>
@@ -12070,7 +12070,7 @@
         <v>Germany</v>
       </c>
       <c r="C285" t="str">
-        <v/>
+        <v>Pforzheim</v>
       </c>
       <c r="D285">
         <v>1925</v>
@@ -12152,7 +12152,7 @@
         <v>Germany</v>
       </c>
       <c r="C287" t="str">
-        <v>Dresden</v>
+        <v>Saxony</v>
       </c>
       <c r="D287" t="str">
         <v/>
@@ -12428,7 +12428,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M293" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>Le Marquand is a Swiss watchmaker based in Bulle, operating under parent company MASTER TIMEKEEPER SA (MTK SA), which merged the André Le Marquand watch company with Side Watch. The brand designs and manufactures watches and watch components for other prestigious labels.</v>
       </c>
     </row>
     <row r="294">
@@ -12685,7 +12685,7 @@
         <v>Italy</v>
       </c>
       <c r="C300" t="str">
-        <v>Elba Island, Italy</v>
+        <v>Marina di Campo</v>
       </c>
       <c r="D300">
         <v>1988</v>
@@ -12892,14 +12892,14 @@
       <c r="C305" t="str">
         <v/>
       </c>
-      <c r="D305" t="str">
-        <v/>
-      </c>
-      <c r="E305" t="str">
-        <v/>
-      </c>
-      <c r="F305" t="str">
-        <v/>
+      <c r="D305">
+        <v>2015</v>
+      </c>
+      <c r="E305">
+        <v>400</v>
+      </c>
+      <c r="F305">
+        <v>1200</v>
       </c>
       <c r="G305" t="str">
         <v>Active</v>
@@ -12914,7 +12914,7 @@
         <v>https://www.louisxvi.de</v>
       </c>
       <c r="K305" t="str">
-        <v/>
+        <v>louisxvi_watches</v>
       </c>
       <c r="L305" t="str">
         <v>MBWDB</v>
@@ -13084,7 +13084,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M309" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>LWC Services is an independent luxury watch service centre based in North Yorkshire, founded by Charlie Walker with over 10 years of industry experience. Specializes in servicing and restoration of Swiss watches including Rolex, Patek Philippe, Audemars Piguet, and Omega. Operates as a boutique buying and servicing experience with trained watchmakers.</v>
       </c>
     </row>
     <row r="310">
@@ -13218,7 +13218,7 @@
         <v>France</v>
       </c>
       <c r="C313" t="str">
-        <v>Paris</v>
+        <v>Reims</v>
       </c>
       <c r="D313" t="str">
         <v/>
@@ -13259,7 +13259,7 @@
         <v>France</v>
       </c>
       <c r="C314" t="str">
-        <v>Paris</v>
+        <v>Lyon</v>
       </c>
       <c r="D314" t="str">
         <v/>
@@ -13423,7 +13423,7 @@
         <v>Germany</v>
       </c>
       <c r="C318" t="str">
-        <v/>
+        <v>Hamburg</v>
       </c>
       <c r="D318">
         <v>2014</v>
@@ -13464,7 +13464,7 @@
         <v>Italy</v>
       </c>
       <c r="C319" t="str">
-        <v>Asti, Italy</v>
+        <v>Asti</v>
       </c>
       <c r="D319" t="str">
         <v/>
@@ -13479,7 +13479,7 @@
         <v>Active</v>
       </c>
       <c r="H319" t="str">
-        <v/>
+        <v>Lunar day</v>
       </c>
       <c r="I319" t="str">
         <v/>
@@ -13488,7 +13488,7 @@
         <v>https://www.marcdarno.com</v>
       </c>
       <c r="K319" t="str">
-        <v/>
+        <v>marcdarno_official</v>
       </c>
       <c r="L319" t="str">
         <v>existing-db</v>
@@ -13710,7 +13710,7 @@
         <v>United Kingdom</v>
       </c>
       <c r="C325" t="str">
-        <v/>
+        <v>London</v>
       </c>
       <c r="D325">
         <v>2015</v>
@@ -13956,7 +13956,7 @@
         <v>Switzerland</v>
       </c>
       <c r="C331" t="str">
-        <v/>
+        <v>Geneva</v>
       </c>
       <c r="D331">
         <v>1886</v>
@@ -14094,7 +14094,7 @@
         <v>Active</v>
       </c>
       <c r="H334" t="str">
-        <v/>
+        <v>ZÜRI-DATE</v>
       </c>
       <c r="I334" t="str">
         <v>2024-01-01</v>
@@ -14325,7 +14325,7 @@
         <v>France</v>
       </c>
       <c r="C340" t="str">
-        <v>Toulouse</v>
+        <v>Bordeaux</v>
       </c>
       <c r="D340" t="str">
         <v/>
@@ -14366,7 +14366,7 @@
         <v>Germany</v>
       </c>
       <c r="C341" t="str">
-        <v/>
+        <v>Münster</v>
       </c>
       <c r="D341">
         <v>2001</v>
@@ -14571,7 +14571,7 @@
         <v>China</v>
       </c>
       <c r="C346" t="str">
-        <v>Pforzheim</v>
+        <v>Beijing</v>
       </c>
       <c r="D346" t="str">
         <v/>
@@ -14650,10 +14650,10 @@
         <v>Micromilspec</v>
       </c>
       <c r="B348" t="str">
-        <v>Switzerland</v>
+        <v>Norway</v>
       </c>
       <c r="C348" t="str">
-        <v>Paris</v>
+        <v>Oslo</v>
       </c>
       <c r="D348" t="str">
         <v/>
@@ -14873,7 +14873,7 @@
         <v>Active</v>
       </c>
       <c r="H353" t="str">
-        <v/>
+        <v>Moduco (First Collection)</v>
       </c>
       <c r="I353" t="str">
         <v>2018-01-24</v>
@@ -15872,7 +15872,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M377" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>Dutch watch brand designed in Amsterdam and made in Europe. Known for the NOWATCH, described as the world's first Awareable analog watch that tracks nervous system health via Reactivity Monitor technology. Offers two main collections: NOWATCH B (comfort-focused) and NOWATCH X (curated craftsmanship).</v>
       </c>
     </row>
     <row r="378">
@@ -16021,10 +16021,10 @@
         <v>Active</v>
       </c>
       <c r="H381" t="str">
-        <v/>
+        <v>Guardian Automatic 36mm</v>
       </c>
       <c r="I381" t="str">
-        <v/>
+        <v>2024-12-19</v>
       </c>
       <c r="J381" t="str">
         <v>https://nordgreen.com/en-us</v>
@@ -16129,7 +16129,7 @@
         <v>Switzerland</v>
       </c>
       <c r="C384" t="str">
-        <v>Bologna</v>
+        <v>La Neuveville</v>
       </c>
       <c r="D384">
         <v>1985</v>
@@ -16252,7 +16252,7 @@
         <v>United Kingdom</v>
       </c>
       <c r="C387" t="str">
-        <v/>
+        <v>London</v>
       </c>
       <c r="D387" t="str">
         <v/>
@@ -16298,11 +16298,11 @@
       <c r="D388">
         <v>2019</v>
       </c>
-      <c r="E388" t="str">
-        <v/>
-      </c>
-      <c r="F388" t="str">
-        <v/>
+      <c r="E388">
+        <v>655</v>
+      </c>
+      <c r="F388">
+        <v>1030</v>
       </c>
       <c r="G388" t="str">
         <v>Active</v>
@@ -16580,7 +16580,7 @@
         <v>United Kingdom</v>
       </c>
       <c r="C395" t="str">
-        <v>Mold</v>
+        <v>Wales</v>
       </c>
       <c r="D395">
         <v>2024</v>
@@ -16700,7 +16700,7 @@
         <v>Palmos</v>
       </c>
       <c r="B398" t="str">
-        <v>United Kingdom</v>
+        <v>Switzerland</v>
       </c>
       <c r="C398" t="str">
         <v>London</v>
@@ -16990,7 +16990,7 @@
         <v>Switzerland</v>
       </c>
       <c r="C405" t="str">
-        <v>La Chaux-de-Fonds</v>
+        <v>Vallée de Joux</v>
       </c>
       <c r="D405">
         <v>2004</v>
@@ -17008,7 +17008,7 @@
         <v>Grandcliff 1004</v>
       </c>
       <c r="I405" t="str">
-        <v/>
+        <v>2024-11-01</v>
       </c>
       <c r="J405" t="str">
         <v>https://www.pierrederoche.com</v>
@@ -17277,7 +17277,7 @@
         <v>Finland</v>
       </c>
       <c r="C412" t="str">
-        <v>Jänsä</v>
+        <v>Joensuu</v>
       </c>
       <c r="D412" t="str">
         <v/>
@@ -17400,7 +17400,7 @@
         <v>Czech Republic</v>
       </c>
       <c r="C415" t="str">
-        <v/>
+        <v>Frýdek-Místek</v>
       </c>
       <c r="D415">
         <v>1949</v>
@@ -17692,11 +17692,11 @@
       <c r="D422" t="str">
         <v/>
       </c>
-      <c r="E422" t="str">
-        <v/>
-      </c>
-      <c r="F422" t="str">
-        <v/>
+      <c r="E422">
+        <v>22</v>
+      </c>
+      <c r="F422">
+        <v>33</v>
       </c>
       <c r="G422" t="str">
         <v>Active</v>
@@ -17848,7 +17848,7 @@
         <v>REC Watches</v>
       </c>
       <c r="B426" t="str">
-        <v>United Kingdom</v>
+        <v>Denmark</v>
       </c>
       <c r="C426" t="str">
         <v/>
@@ -17963,7 +17963,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M428" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>Reloj.es is a Spanish watch retailer specializing in men's watches (Relojes Para Hombres). Part of Holland Watch Group B.V., the site operates as a multi-brand distributor carrying 70+ watch brands rather than as an independent watch manufacturer.</v>
       </c>
     </row>
     <row r="429">
@@ -18184,17 +18184,17 @@
       <c r="D434" t="str">
         <v/>
       </c>
-      <c r="E434" t="str">
-        <v/>
-      </c>
-      <c r="F434" t="str">
-        <v/>
+      <c r="E434">
+        <v>302</v>
+      </c>
+      <c r="F434">
+        <v>1670</v>
       </c>
       <c r="G434" t="str">
         <v>Active</v>
       </c>
       <c r="H434" t="str">
-        <v/>
+        <v>CHAPTER 3</v>
       </c>
       <c r="I434" t="str">
         <v/>
@@ -18203,7 +18203,7 @@
         <v>https://riskers-watches.com/</v>
       </c>
       <c r="K434" t="str">
-        <v/>
+        <v>riskers_watches</v>
       </c>
       <c r="L434" t="str">
         <v>MBWDB</v>
@@ -18425,7 +18425,7 @@
         <v>Switzerland</v>
       </c>
       <c r="C440" t="str">
-        <v/>
+        <v>La Chaux-de-Fonds</v>
       </c>
       <c r="D440">
         <v>1895</v>
@@ -18712,7 +18712,7 @@
         <v>Italy</v>
       </c>
       <c r="C447" t="str">
-        <v/>
+        <v>Florence</v>
       </c>
       <c r="D447">
         <v>1927</v>
@@ -18835,7 +18835,7 @@
         <v>Switzerland</v>
       </c>
       <c r="C450" t="str">
-        <v>Le Locle</v>
+        <v>Alle</v>
       </c>
       <c r="D450" t="str">
         <v/>
@@ -18917,7 +18917,7 @@
         <v>United Kingdom</v>
       </c>
       <c r="C452" t="str">
-        <v/>
+        <v>London</v>
       </c>
       <c r="D452">
         <v>2014</v>
@@ -19250,11 +19250,11 @@
       <c r="D460">
         <v>2019</v>
       </c>
-      <c r="E460" t="str">
-        <v/>
-      </c>
-      <c r="F460" t="str">
-        <v/>
+      <c r="E460">
+        <v>400</v>
+      </c>
+      <c r="F460">
+        <v>800</v>
       </c>
       <c r="G460" t="str">
         <v>Active</v>
@@ -19269,7 +19269,7 @@
         <v>https://www.serica.watch</v>
       </c>
       <c r="K460" t="str">
-        <v/>
+        <v>serica_watches</v>
       </c>
       <c r="L460" t="str">
         <v>existing-db</v>
@@ -19491,7 +19491,7 @@
         <v>Germany</v>
       </c>
       <c r="C466" t="str">
-        <v>Frankfurt</v>
+        <v>Frankfurt am Main</v>
       </c>
       <c r="D466">
         <v>1961</v>
@@ -19767,7 +19767,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M472" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>Swedish watch brand exclusively dedicated to rectangular and square case watches. Offers four main collections: Legacy (3-year battery), Nostalgia (11-year battery), Momentum (self-winding), and Amorous (self-winding). Backed by 10-year warranty and available in multiple case finishes and dial colors.</v>
       </c>
     </row>
     <row r="473">
@@ -19901,7 +19901,7 @@
         <v>Switzerland</v>
       </c>
       <c r="C476" t="str">
-        <v>Neuchâtel</v>
+        <v>Geneva</v>
       </c>
       <c r="D476">
         <v>2002</v>
@@ -20062,10 +20062,10 @@
         <v>Steinhart</v>
       </c>
       <c r="B480" t="str">
-        <v>Switzerland</v>
+        <v>Germany</v>
       </c>
       <c r="C480" t="str">
-        <v/>
+        <v>Hamburg</v>
       </c>
       <c r="D480">
         <v>2001</v>
@@ -20188,7 +20188,7 @@
         <v>Germany</v>
       </c>
       <c r="C483" t="str">
-        <v/>
+        <v>Pforzheim</v>
       </c>
       <c r="D483">
         <v>1927</v>
@@ -20431,7 +20431,7 @@
         <v>Subdelta</v>
       </c>
       <c r="B489" t="str">
-        <v>Germany</v>
+        <v>Netherlands</v>
       </c>
       <c r="C489" t="str">
         <v>Hengelo</v>
@@ -20721,7 +20721,7 @@
         <v>United Kingdom</v>
       </c>
       <c r="C496" t="str">
-        <v>Southwell</v>
+        <v>London</v>
       </c>
       <c r="D496" t="str">
         <v/>
@@ -20759,10 +20759,10 @@
         <v>Techne Instruments</v>
       </c>
       <c r="B497" t="str">
-        <v>Sweden</v>
+        <v>United States</v>
       </c>
       <c r="C497" t="str">
-        <v/>
+        <v>Berkeley</v>
       </c>
       <c r="D497">
         <v>2007</v>
@@ -20967,7 +20967,7 @@
         <v>Germany</v>
       </c>
       <c r="C502" t="str">
-        <v/>
+        <v>Munich</v>
       </c>
       <c r="D502">
         <v>2004</v>
@@ -21054,11 +21054,11 @@
       <c r="D504" t="str">
         <v/>
       </c>
-      <c r="E504" t="str">
-        <v/>
-      </c>
-      <c r="F504" t="str">
-        <v/>
+      <c r="E504">
+        <v>1015</v>
+      </c>
+      <c r="F504">
+        <v>1585</v>
       </c>
       <c r="G504" t="str">
         <v>Active</v>
@@ -21073,7 +21073,7 @@
         <v>https://timeless-watch.ch/</v>
       </c>
       <c r="K504" t="str">
-        <v/>
+        <v>timeless.swiss.watch</v>
       </c>
       <c r="L504" t="str">
         <v>MBWDB</v>
@@ -21087,7 +21087,7 @@
         <v>Tissel</v>
       </c>
       <c r="B505" t="str">
-        <v>South Korea</v>
+        <v>Czech Republic</v>
       </c>
       <c r="C505" t="str">
         <v/>
@@ -21128,7 +21128,7 @@
         <v>Titus Watches</v>
       </c>
       <c r="B506" t="str">
-        <v>Switzerland</v>
+        <v>Hong Kong</v>
       </c>
       <c r="C506" t="str">
         <v/>
@@ -21272,7 +21272,7 @@
         <v>P96 OdP Color</v>
       </c>
       <c r="I509" t="str">
-        <v/>
+        <v>2024-01-01</v>
       </c>
       <c r="J509" t="str">
         <v>https://www.traser.ch</v>
@@ -21295,7 +21295,7 @@
         <v>Germany</v>
       </c>
       <c r="C510" t="str">
-        <v/>
+        <v>Hamburg</v>
       </c>
       <c r="D510">
         <v>2014</v>
@@ -21459,16 +21459,16 @@
         <v>Germany</v>
       </c>
       <c r="C514" t="str">
-        <v>Evanston</v>
-      </c>
-      <c r="D514" t="str">
-        <v/>
-      </c>
-      <c r="E514" t="str">
-        <v/>
-      </c>
-      <c r="F514" t="str">
-        <v/>
+        <v>Munich</v>
+      </c>
+      <c r="D514">
+        <v>1828</v>
+      </c>
+      <c r="E514">
+        <v>289</v>
+      </c>
+      <c r="F514">
+        <v>2265</v>
       </c>
       <c r="G514" t="str">
         <v>Active</v>
@@ -21483,7 +21483,7 @@
         <v>https://tufinawatches.com/</v>
       </c>
       <c r="K514" t="str">
-        <v/>
+        <v>tufina_watches</v>
       </c>
       <c r="L514" t="str">
         <v>MBWDB</v>
@@ -21770,7 +21770,7 @@
         <v>https://ugolinimeccanicawatches.com/</v>
       </c>
       <c r="K521" t="str">
-        <v/>
+        <v>ugolinimeccanicawatches</v>
       </c>
       <c r="L521" t="str">
         <v>MBWDB</v>
@@ -21787,7 +21787,7 @@
         <v>Hong Kong</v>
       </c>
       <c r="C522" t="str">
-        <v/>
+        <v>Hong Kong</v>
       </c>
       <c r="D522">
         <v>2014</v>
@@ -21828,7 +21828,7 @@
         <v>Italy</v>
       </c>
       <c r="C523" t="str">
-        <v/>
+        <v>Milan</v>
       </c>
       <c r="D523">
         <v>2015</v>
@@ -21869,7 +21869,7 @@
         <v>Germany</v>
       </c>
       <c r="C524" t="str">
-        <v>Munich</v>
+        <v>Holzkirchen</v>
       </c>
       <c r="D524" t="str">
         <v/>
@@ -21915,11 +21915,11 @@
       <c r="D525" t="str">
         <v/>
       </c>
-      <c r="E525" t="str">
-        <v/>
-      </c>
-      <c r="F525" t="str">
-        <v/>
+      <c r="E525">
+        <v>349</v>
+      </c>
+      <c r="F525">
+        <v>809</v>
       </c>
       <c r="G525" t="str">
         <v>Active</v>
@@ -21934,7 +21934,7 @@
         <v>https://www.valhallaofnorway.no/</v>
       </c>
       <c r="K525" t="str">
-        <v/>
+        <v>valhallawatches</v>
       </c>
       <c r="L525" t="str">
         <v>MBWDB</v>
@@ -22637,7 +22637,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M542" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>Norwegian watch brand creating timeless wristwatches inspired by Norwegian nature, culture and history. Designs are made in Norway with Swiss movements. Collections include Tandberg, URÆD GMT, Runde, and special editions like Norway Chess collaboration.</v>
       </c>
     </row>
     <row r="543">
@@ -22689,7 +22689,7 @@
         <v>Lithuania</v>
       </c>
       <c r="C544" t="str">
-        <v/>
+        <v>Vilnius</v>
       </c>
       <c r="D544">
         <v>2003</v>
@@ -22730,7 +22730,7 @@
         <v>Russia</v>
       </c>
       <c r="C545" t="str">
-        <v/>
+        <v>Chistopol</v>
       </c>
       <c r="D545" t="str">
         <v/>
@@ -22738,8 +22738,8 @@
       <c r="E545" t="str">
         <v/>
       </c>
-      <c r="F545" t="str">
-        <v/>
+      <c r="F545">
+        <v>606</v>
       </c>
       <c r="G545" t="str">
         <v>Active</v>
@@ -22894,7 +22894,7 @@
         <v>United States</v>
       </c>
       <c r="C549" t="str">
-        <v/>
+        <v>Meriden</v>
       </c>
       <c r="D549">
         <v>1978</v>
@@ -22912,7 +22912,7 @@
         <v>Heritage Sportline</v>
       </c>
       <c r="I549" t="str">
-        <v/>
+        <v>2024-01-01</v>
       </c>
       <c r="J549" t="str">
         <v>https://delraywatch.com/waldan-international-1/</v>
@@ -22935,7 +22935,7 @@
         <v>Poland</v>
       </c>
       <c r="C550" t="str">
-        <v/>
+        <v>Warsaw</v>
       </c>
       <c r="D550" t="str">
         <v/>
@@ -23304,7 +23304,7 @@
         <v>France</v>
       </c>
       <c r="C559" t="str">
-        <v/>
+        <v>Morteau</v>
       </c>
       <c r="D559">
         <v>1948</v>
@@ -23629,7 +23629,7 @@
         <v>Zlatoust</v>
       </c>
       <c r="B567" t="str">
-        <v>Soviet Union</v>
+        <v>Russia</v>
       </c>
       <c r="C567" t="str">
         <v>Zlatoust</v>
@@ -23675,8 +23675,8 @@
       <c r="C568" t="str">
         <v>Zlatoust</v>
       </c>
-      <c r="D568" t="str">
-        <v/>
+      <c r="D568">
+        <v>1947</v>
       </c>
       <c r="E568" t="str">
         <v/>
@@ -24221,7 +24221,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M11" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>No homepage content provided for data extraction. Unable to verify current status or details for ARETHUSA Watch Company.</v>
       </c>
     </row>
     <row r="12">
@@ -24847,16 +24847,16 @@
         <v>United States</v>
       </c>
       <c r="C27" t="str">
-        <v>Bern</v>
+        <v>Denver</v>
       </c>
       <c r="D27">
         <v>2016</v>
       </c>
-      <c r="E27" t="str">
-        <v/>
-      </c>
-      <c r="F27" t="str">
-        <v/>
+      <c r="E27">
+        <v>495</v>
+      </c>
+      <c r="F27">
+        <v>695</v>
       </c>
       <c r="G27" t="str">
         <v>Active</v>
@@ -24871,7 +24871,7 @@
         <v>https://bernwatches.com</v>
       </c>
       <c r="K27" t="str">
-        <v/>
+        <v>bernwatch</v>
       </c>
       <c r="L27" t="str">
         <v>MBWDB</v>
@@ -24929,7 +24929,7 @@
         <v>United States</v>
       </c>
       <c r="C29" t="str">
-        <v/>
+        <v>Cuyahoga Falls</v>
       </c>
       <c r="D29">
         <v>1990</v>
@@ -25328,7 +25328,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M38" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>California Watch Co. designs timepieces with attention to dimensional details including concave subdials, raised indices, and domed dials. The brand offers diverse collections including PCH Driver Jump Hour, Venice Beach Digital, and chronograph models. Currently carries 42 products ranging from $79.99 to $149.99.</v>
       </c>
     </row>
     <row r="39">
@@ -25503,7 +25503,7 @@
         <v>Chile</v>
       </c>
       <c r="C43" t="str">
-        <v/>
+        <v>Valparaíso</v>
       </c>
       <c r="D43" t="str">
         <v/>
@@ -25585,7 +25585,7 @@
         <v>United States</v>
       </c>
       <c r="C45" t="str">
-        <v/>
+        <v>Denver</v>
       </c>
       <c r="D45">
         <v>2009</v>
@@ -25623,19 +25623,19 @@
         <v>Chase-Durer Watch Company</v>
       </c>
       <c r="B46" t="str">
-        <v>USA</v>
+        <v>United States</v>
       </c>
       <c r="C46" t="str">
-        <v>Los Angeles, California</v>
-      </c>
-      <c r="D46" t="str">
-        <v/>
-      </c>
-      <c r="E46" t="str">
-        <v/>
-      </c>
-      <c r="F46" t="str">
-        <v/>
+        <v>Houston</v>
+      </c>
+      <c r="D46">
+        <v>1988</v>
+      </c>
+      <c r="E46">
+        <v>1200</v>
+      </c>
+      <c r="F46">
+        <v>2800</v>
       </c>
       <c r="G46" t="str">
         <v>Active</v>
@@ -25650,7 +25650,7 @@
         <v>https://www.chase-durer.com</v>
       </c>
       <c r="K46" t="str">
-        <v/>
+        <v>chasedurer</v>
       </c>
       <c r="L46" t="str">
         <v>existing-db</v>
@@ -25669,8 +25669,8 @@
       <c r="C47" t="str">
         <v>Cincinnati</v>
       </c>
-      <c r="D47" t="str">
-        <v/>
+      <c r="D47">
+        <v>1869</v>
       </c>
       <c r="E47" t="str">
         <v/>
@@ -25808,7 +25808,7 @@
         <v>MILLENIUM</v>
       </c>
       <c r="I50" t="str">
-        <v/>
+        <v>2024-12-01</v>
       </c>
       <c r="J50" t="str">
         <v>https://www.crotonwatch.com</v>
@@ -25915,14 +25915,14 @@
       <c r="C53" t="str">
         <v>Los Angeles</v>
       </c>
-      <c r="D53" t="str">
-        <v/>
-      </c>
-      <c r="E53" t="str">
-        <v/>
-      </c>
-      <c r="F53" t="str">
-        <v/>
+      <c r="D53">
+        <v>2009</v>
+      </c>
+      <c r="E53">
+        <v>5000</v>
+      </c>
+      <c r="F53">
+        <v>50000</v>
       </c>
       <c r="G53" t="str">
         <v>Active</v>
@@ -26010,10 +26010,10 @@
         <v>Active</v>
       </c>
       <c r="H55" t="str">
-        <v/>
+        <v>Seiko Yachtmaster Stealth Mod</v>
       </c>
       <c r="I55" t="str">
-        <v/>
+        <v>2024-07-17</v>
       </c>
       <c r="J55" t="str">
         <v>https://www.dagazwatch.com</v>
@@ -26077,7 +26077,7 @@
         <v>United States</v>
       </c>
       <c r="C57" t="str">
-        <v>Dallas</v>
+        <v>Texas</v>
       </c>
       <c r="D57" t="str">
         <v/>
@@ -26118,7 +26118,7 @@
         <v>United States</v>
       </c>
       <c r="C58" t="str">
-        <v/>
+        <v>New York</v>
       </c>
       <c r="D58">
         <v>2007</v>
@@ -26279,10 +26279,10 @@
         <v>Draken</v>
       </c>
       <c r="B62" t="str">
-        <v>United States</v>
+        <v>New Zealand</v>
       </c>
       <c r="C62" t="str">
-        <v/>
+        <v>Waipu</v>
       </c>
       <c r="D62" t="str">
         <v/>
@@ -26435,7 +26435,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M65" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>Duxot was a watch brand under Dartmouth Brands in the United States. Limited reliable information available in training data. Brand appears to be inactive or defunct.</v>
       </c>
     </row>
     <row r="66">
@@ -26446,7 +26446,7 @@
         <v>United States</v>
       </c>
       <c r="C66" t="str">
-        <v>Hagerstown</v>
+        <v>Baltimore</v>
       </c>
       <c r="D66" t="str">
         <v/>
@@ -26569,7 +26569,7 @@
         <v>United States</v>
       </c>
       <c r="C69" t="str">
-        <v/>
+        <v>San Francisco</v>
       </c>
       <c r="D69">
         <v>2012</v>
@@ -26774,7 +26774,7 @@
         <v>United States</v>
       </c>
       <c r="C74" t="str">
-        <v/>
+        <v>Antelope</v>
       </c>
       <c r="D74" t="str">
         <v/>
@@ -26804,7 +26804,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M74" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>Famine Studios is a US-based brand based in Antelope, California. The company primarily sells apparel and accessories, with limited watch offerings including the Moneyman Watch. Brand is currently active with an ongoing sweepstakes promotion (September-December 2025).</v>
       </c>
     </row>
     <row r="75">
@@ -26815,7 +26815,7 @@
         <v>United States</v>
       </c>
       <c r="C75" t="str">
-        <v>Elmhurst</v>
+        <v>Chicago</v>
       </c>
       <c r="D75" t="str">
         <v/>
@@ -27158,7 +27158,7 @@
         <v>Active</v>
       </c>
       <c r="H83" t="str">
-        <v/>
+        <v>Windmaster</v>
       </c>
       <c r="I83" t="str">
         <v/>
@@ -27230,11 +27230,11 @@
       <c r="D85" t="str">
         <v/>
       </c>
-      <c r="E85" t="str">
-        <v/>
-      </c>
-      <c r="F85" t="str">
-        <v/>
+      <c r="E85">
+        <v>864</v>
+      </c>
+      <c r="F85">
+        <v>2227</v>
       </c>
       <c r="G85" t="str">
         <v>Active</v>
@@ -27249,7 +27249,7 @@
         <v>https://grandeur-usa.com/</v>
       </c>
       <c r="K85" t="str">
-        <v/>
+        <v>grandeur</v>
       </c>
       <c r="L85" t="str">
         <v>MBWDB</v>
@@ -27430,7 +27430,7 @@
         <v>Canada</v>
       </c>
       <c r="C90" t="str">
-        <v/>
+        <v>Toronto</v>
       </c>
       <c r="D90">
         <v>2015</v>
@@ -27473,14 +27473,14 @@
       <c r="C91" t="str">
         <v/>
       </c>
-      <c r="D91" t="str">
-        <v/>
-      </c>
-      <c r="E91" t="str">
-        <v/>
-      </c>
-      <c r="F91" t="str">
-        <v/>
+      <c r="D91">
+        <v>2012</v>
+      </c>
+      <c r="E91">
+        <v>295</v>
+      </c>
+      <c r="F91">
+        <v>595</v>
       </c>
       <c r="G91" t="str">
         <v>Active</v>
@@ -27495,7 +27495,7 @@
         <v>https://www.helmwatches.com</v>
       </c>
       <c r="K91" t="str">
-        <v/>
+        <v>helmwatches</v>
       </c>
       <c r="L91" t="str">
         <v>MBWDB</v>
@@ -27594,7 +27594,7 @@
         <v>United States</v>
       </c>
       <c r="C94" t="str">
-        <v>Brooklyn</v>
+        <v>New York</v>
       </c>
       <c r="D94" t="str">
         <v/>
@@ -27804,11 +27804,11 @@
       <c r="D99">
         <v>2019</v>
       </c>
-      <c r="E99" t="str">
-        <v/>
-      </c>
-      <c r="F99" t="str">
-        <v/>
+      <c r="E99">
+        <v>195</v>
+      </c>
+      <c r="F99">
+        <v>395</v>
       </c>
       <c r="G99" t="str">
         <v>Active</v>
@@ -27878,10 +27878,10 @@
         <v>JEAN VERNIER</v>
       </c>
       <c r="B101" t="str">
-        <v>Brazil</v>
+        <v>United States</v>
       </c>
       <c r="C101" t="str">
-        <v>Rio de Janeiro</v>
+        <v>New York</v>
       </c>
       <c r="D101">
         <v>1991</v>
@@ -28004,7 +28004,7 @@
         <v>United States</v>
       </c>
       <c r="C104" t="str">
-        <v>Washington, DC</v>
+        <v>Washington, D.C.</v>
       </c>
       <c r="D104" t="str">
         <v/>
@@ -28086,7 +28086,7 @@
         <v>United States</v>
       </c>
       <c r="C106" t="str">
-        <v>Washington DC</v>
+        <v>Washington, D.C.</v>
       </c>
       <c r="D106" t="str">
         <v/>
@@ -28104,7 +28104,7 @@
         <v>Round Signature Shades</v>
       </c>
       <c r="I106" t="str">
-        <v/>
+        <v>2021-12-31</v>
       </c>
       <c r="J106" t="str">
         <v>https://www.kjosephwatches.com/</v>
@@ -28198,7 +28198,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M108" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>Canadian microbrand based in Montreal. Specializes in automatic GMT watches designed for global travelers. Watches are hand-assembled and tested in Montreal with Miyota 9075 Japanese movements and 24-month warranty.</v>
       </c>
     </row>
     <row r="109">
@@ -28580,14 +28580,14 @@
       <c r="C118" t="str">
         <v/>
       </c>
-      <c r="D118" t="str">
-        <v/>
-      </c>
-      <c r="E118" t="str">
-        <v/>
-      </c>
-      <c r="F118" t="str">
-        <v/>
+      <c r="D118">
+        <v>2007</v>
+      </c>
+      <c r="E118">
+        <v>295</v>
+      </c>
+      <c r="F118">
+        <v>595</v>
       </c>
       <c r="G118" t="str">
         <v>Active</v>
@@ -28602,7 +28602,7 @@
         <v>https://www.maratac.com</v>
       </c>
       <c r="K118" t="str">
-        <v/>
+        <v>maratac</v>
       </c>
       <c r="L118" t="str">
         <v>MBWDB</v>
@@ -28783,7 +28783,7 @@
         <v>United States</v>
       </c>
       <c r="C123" t="str">
-        <v/>
+        <v>Chenoa</v>
       </c>
       <c r="D123">
         <v>2017</v>
@@ -29029,7 +29029,7 @@
         <v>United States</v>
       </c>
       <c r="C129" t="str">
-        <v>North Carolina</v>
+        <v>Charlotte</v>
       </c>
       <c r="D129" t="str">
         <v/>
@@ -29272,7 +29272,7 @@
         <v>Nodus Watches</v>
       </c>
       <c r="B135" t="str">
-        <v>USA</v>
+        <v>United States</v>
       </c>
       <c r="C135" t="str">
         <v>Los Angeles</v>
@@ -29357,7 +29357,7 @@
         <v>United States</v>
       </c>
       <c r="C137" t="str">
-        <v/>
+        <v>Portland</v>
       </c>
       <c r="D137">
         <v>2017</v>
@@ -29480,7 +29480,7 @@
         <v>Hong Kong</v>
       </c>
       <c r="C140" t="str">
-        <v/>
+        <v>Hong Kong</v>
       </c>
       <c r="D140" t="str">
         <v/>
@@ -29879,7 +29879,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M149" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>US-based microbrand assembling adventure-ready field watches. Cascadia Field Watch features 316L stainless steel case, sapphire crystal, Ameriquartz movement with 5-year warranty, and 100m water resistance. Emphasizes slow goods philosophy with American assembly and quick-release strap system.</v>
       </c>
     </row>
     <row r="150">
@@ -30056,14 +30056,14 @@
       <c r="C154" t="str">
         <v/>
       </c>
-      <c r="D154" t="str">
-        <v/>
-      </c>
-      <c r="E154" t="str">
-        <v/>
-      </c>
-      <c r="F154" t="str">
-        <v/>
+      <c r="D154">
+        <v>2010</v>
+      </c>
+      <c r="E154">
+        <v>295</v>
+      </c>
+      <c r="F154">
+        <v>595</v>
       </c>
       <c r="G154" t="str">
         <v>Active</v>
@@ -30177,7 +30177,7 @@
         <v>United States</v>
       </c>
       <c r="C157" t="str">
-        <v/>
+        <v>Agoura Hills</v>
       </c>
       <c r="D157">
         <v>2017</v>
@@ -30505,7 +30505,7 @@
         <v>United States</v>
       </c>
       <c r="C165" t="str">
-        <v/>
+        <v>Lancaster</v>
       </c>
       <c r="D165">
         <v>1992</v>
@@ -30874,7 +30874,7 @@
         <v>Puerto Rico</v>
       </c>
       <c r="C174" t="str">
-        <v>San Juan</v>
+        <v>Santurce</v>
       </c>
       <c r="D174" t="str">
         <v/>
@@ -31381,16 +31381,16 @@
         <v>Active</v>
       </c>
       <c r="H186" t="str">
-        <v/>
+        <v>Speidel x Life Is Good Watches</v>
       </c>
       <c r="I186" t="str">
-        <v/>
+        <v>2026-01-01</v>
       </c>
       <c r="J186" t="str">
         <v>https://www.speidel.com</v>
       </c>
       <c r="K186" t="str">
-        <v/>
+        <v>speidel1904</v>
       </c>
       <c r="L186" t="str">
         <v>MBWDB</v>
@@ -31876,7 +31876,7 @@
         <v>TIME BOLD - CX2</v>
       </c>
       <c r="I198" t="str">
-        <v/>
+        <v>2024-12-01</v>
       </c>
       <c r="J198" t="str">
         <v>https://torinocarrero.com/</v>
@@ -31888,7 +31888,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M198" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>Torino Carrero is a US-based watch brand based in Encino, California. The brand offers diverse collections including automatic, quartz, chronograph, and multi-function watches for men and women, with models like Catania, Milazo, Avatar, and Gem Master series. Known for sport and diving watches with prices ranging from approximately $1,900 to $3,200.</v>
       </c>
     </row>
     <row r="199">
@@ -31899,10 +31899,10 @@
         <v>United States</v>
       </c>
       <c r="C199" t="str">
-        <v/>
-      </c>
-      <c r="D199" t="str">
-        <v/>
+        <v>New York</v>
+      </c>
+      <c r="D199">
+        <v>1993</v>
       </c>
       <c r="E199">
         <v>99</v>
@@ -31917,13 +31917,13 @@
         <v>TR-660</v>
       </c>
       <c r="I199" t="str">
-        <v/>
+        <v>2024-08-15</v>
       </c>
       <c r="J199" t="str">
         <v>https://www.tornekrayville.com</v>
       </c>
       <c r="K199" t="str">
-        <v/>
+        <v>tornekrayville</v>
       </c>
       <c r="L199" t="str">
         <v>MBWDB</v>
@@ -32019,7 +32019,7 @@
         <v>Trintec</v>
       </c>
       <c r="B202" t="str">
-        <v>United States</v>
+        <v>Canada</v>
       </c>
       <c r="C202" t="str">
         <v/>
@@ -32040,7 +32040,7 @@
         <v>CoPilot GMT</v>
       </c>
       <c r="I202" t="str">
-        <v/>
+        <v>2024-12-31</v>
       </c>
       <c r="J202" t="str">
         <v>https://www.trintecwatches.com</v>
@@ -32347,7 +32347,7 @@
         <v>VeriWatch</v>
       </c>
       <c r="B210" t="str">
-        <v>Italy</v>
+        <v>United States</v>
       </c>
       <c r="C210" t="str">
         <v/>
@@ -32432,7 +32432,7 @@
         <v>United States</v>
       </c>
       <c r="C212" t="str">
-        <v/>
+        <v>Austin</v>
       </c>
       <c r="D212">
         <v>2014</v>
@@ -32924,7 +32924,7 @@
         <v>United States</v>
       </c>
       <c r="C224" t="str">
-        <v/>
+        <v>Los Angeles</v>
       </c>
       <c r="D224">
         <v>2012</v>
@@ -33006,7 +33006,7 @@
         <v>Brazil</v>
       </c>
       <c r="C226" t="str">
-        <v>Rio</v>
+        <v>São Paulo</v>
       </c>
       <c r="D226" t="str">
         <v/>
@@ -33047,7 +33047,7 @@
         <v>Singapore</v>
       </c>
       <c r="C227" t="str">
-        <v/>
+        <v>Singapore</v>
       </c>
       <c r="D227">
         <v>2014</v>
@@ -33196,7 +33196,7 @@
         <v>Hong Kong</v>
       </c>
       <c r="C3" t="str">
-        <v>Hong Kong</v>
+        <v>Kowloon</v>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -33319,7 +33319,7 @@
         <v>Netherlands</v>
       </c>
       <c r="C6" t="str">
-        <v/>
+        <v>Horst</v>
       </c>
       <c r="D6" t="str">
         <v/>
@@ -33524,7 +33524,7 @@
         <v>China</v>
       </c>
       <c r="C11" t="str">
-        <v>Singapore, Singapore</v>
+        <v>Hong Kong</v>
       </c>
       <c r="D11" t="str">
         <v/>
@@ -33565,7 +33565,7 @@
         <v>Indonesia</v>
       </c>
       <c r="C12" t="str">
-        <v/>
+        <v>Jakarta</v>
       </c>
       <c r="D12" t="str">
         <v/>
@@ -33624,7 +33624,7 @@
         <v>Ettore Drift</v>
       </c>
       <c r="I13" t="str">
-        <v/>
+        <v>2024-12-23</v>
       </c>
       <c r="J13" t="str">
         <v>https://www.atowak.com</v>
@@ -33688,7 +33688,7 @@
         <v>Hong Kong</v>
       </c>
       <c r="C15" t="str">
-        <v/>
+        <v>Hong Kong</v>
       </c>
       <c r="D15">
         <v>2010</v>
@@ -33729,7 +33729,7 @@
         <v>China</v>
       </c>
       <c r="C16" t="str">
-        <v/>
+        <v>Dongguan</v>
       </c>
       <c r="D16" t="str">
         <v/>
@@ -34062,11 +34062,11 @@
       <c r="D24">
         <v>1993</v>
       </c>
-      <c r="E24" t="str">
-        <v/>
-      </c>
-      <c r="F24" t="str">
-        <v/>
+      <c r="E24">
+        <v>19</v>
+      </c>
+      <c r="F24">
+        <v>175</v>
       </c>
       <c r="G24" t="str">
         <v>Active</v>
@@ -34081,7 +34081,7 @@
         <v>https://bureiwatches.com/</v>
       </c>
       <c r="K24" t="str">
-        <v/>
+        <v>bureiwatches</v>
       </c>
       <c r="L24" t="str">
         <v>MBWDB</v>
@@ -34267,11 +34267,11 @@
       <c r="D29">
         <v>2019</v>
       </c>
-      <c r="E29" t="str">
-        <v/>
-      </c>
-      <c r="F29" t="str">
-        <v/>
+      <c r="E29">
+        <v>2200</v>
+      </c>
+      <c r="F29">
+        <v>2500</v>
       </c>
       <c r="G29" t="str">
         <v>Active</v>
@@ -34286,7 +34286,7 @@
         <v>https://linkandtag.com/2025/10/18/ckl-watches/</v>
       </c>
       <c r="K29" t="str">
-        <v/>
+        <v>linkandtag2017</v>
       </c>
       <c r="L29" t="str">
         <v>MBWDB</v>
@@ -34308,11 +34308,11 @@
       <c r="D30" t="str">
         <v/>
       </c>
-      <c r="E30" t="str">
-        <v/>
-      </c>
-      <c r="F30" t="str">
-        <v/>
+      <c r="E30">
+        <v>153</v>
+      </c>
+      <c r="F30">
+        <v>228</v>
       </c>
       <c r="G30" t="str">
         <v>Active</v>
@@ -34327,7 +34327,7 @@
         <v>https://corgeutwatchco.com/</v>
       </c>
       <c r="K30" t="str">
-        <v/>
+        <v>corgeut_watches</v>
       </c>
       <c r="L30" t="str">
         <v>MBWDB</v>
@@ -34795,7 +34795,7 @@
         <v>Singapore</v>
       </c>
       <c r="C42" t="str">
-        <v>Geylang</v>
+        <v>Singapore</v>
       </c>
       <c r="D42" t="str">
         <v/>
@@ -34877,10 +34877,10 @@
         <v>China</v>
       </c>
       <c r="C44" t="str">
-        <v/>
-      </c>
-      <c r="D44" t="str">
-        <v/>
+        <v>Foshan</v>
+      </c>
+      <c r="D44">
+        <v>1989</v>
       </c>
       <c r="E44" t="str">
         <v/>
@@ -34895,7 +34895,7 @@
         <v/>
       </c>
       <c r="I44" t="str">
-        <v/>
+        <v>2025-01-01</v>
       </c>
       <c r="J44" t="str">
         <v>https://guanqin-watch.com/</v>
@@ -35082,7 +35082,7 @@
         <v>India</v>
       </c>
       <c r="C49" t="str">
-        <v/>
+        <v>Bangalore</v>
       </c>
       <c r="D49">
         <v>1949</v>
@@ -35393,7 +35393,7 @@
         <v>https://jaipur.watch/en-us</v>
       </c>
       <c r="K56" t="str">
-        <v/>
+        <v>jaipurwatchcompany</v>
       </c>
       <c r="L56" t="str">
         <v>MBWDB</v>
@@ -35410,7 +35410,7 @@
         <v>Singapore</v>
       </c>
       <c r="C57" t="str">
-        <v/>
+        <v>Singapore</v>
       </c>
       <c r="D57" t="str">
         <v/>
@@ -35507,10 +35507,10 @@
         <v>Active</v>
       </c>
       <c r="H59" t="str">
-        <v/>
+        <v>Classic Standard</v>
       </c>
       <c r="I59" t="str">
-        <v/>
+        <v>2024-09-30</v>
       </c>
       <c r="J59" t="str">
         <v>http://www.kentexwatch.com/</v>
@@ -35533,16 +35533,16 @@
         <v>Japan</v>
       </c>
       <c r="C60" t="str">
-        <v>Asakusa</v>
+        <v>Tokyo</v>
       </c>
       <c r="D60">
         <v>2025</v>
       </c>
-      <c r="E60" t="str">
-        <v/>
-      </c>
-      <c r="F60" t="str">
-        <v/>
+      <c r="E60">
+        <v>650</v>
+      </c>
+      <c r="F60">
+        <v>690</v>
       </c>
       <c r="G60" t="str">
         <v>Active</v>
@@ -35557,7 +35557,7 @@
         <v>https://kiwametokyo.com/en/collections/watches</v>
       </c>
       <c r="K60" t="str">
-        <v/>
+        <v>kiwametokyo</v>
       </c>
       <c r="L60" t="str">
         <v>MBWDB</v>
@@ -35620,17 +35620,17 @@
       <c r="D62">
         <v>2020</v>
       </c>
-      <c r="E62" t="str">
-        <v/>
-      </c>
-      <c r="F62" t="str">
-        <v/>
+      <c r="E62">
+        <v>596</v>
+      </c>
+      <c r="F62">
+        <v>889</v>
       </c>
       <c r="G62" t="str">
         <v>Active</v>
       </c>
       <c r="H62" t="str">
-        <v/>
+        <v>ROYAL SMITH 90-010</v>
       </c>
       <c r="I62" t="str">
         <v>2026-04-04</v>
@@ -36096,7 +36096,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M73" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>KENKO Mayonnaise is a Japanese food company, not a watch brand. The homepage and provided content relate to mayonnaise and salad dressing products, not timepieces.</v>
       </c>
     </row>
     <row r="74">
@@ -36115,8 +36115,8 @@
       <c r="E74">
         <v>600</v>
       </c>
-      <c r="F74" t="str">
-        <v/>
+      <c r="F74">
+        <v>800</v>
       </c>
       <c r="G74" t="str">
         <v>Active</v>
@@ -36131,7 +36131,7 @@
         <v>https://www.melbournewatchco.com</v>
       </c>
       <c r="K74" t="str">
-        <v/>
+        <v>melbournewatchco</v>
       </c>
       <c r="L74" t="str">
         <v>MBWDB</v>
@@ -36153,11 +36153,11 @@
       <c r="D75">
         <v>2013</v>
       </c>
-      <c r="E75" t="str">
-        <v/>
-      </c>
-      <c r="F75" t="str">
-        <v/>
+      <c r="E75">
+        <v>400</v>
+      </c>
+      <c r="F75">
+        <v>800</v>
       </c>
       <c r="G75" t="str">
         <v>Active</v>
@@ -36172,7 +36172,7 @@
         <v>https://www.melbournewatchco.com</v>
       </c>
       <c r="K75" t="str">
-        <v/>
+        <v>melbournewatchcompany</v>
       </c>
       <c r="L75" t="str">
         <v>MBWDB</v>
@@ -36219,7 +36219,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M76" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>Singapore-based microbrand founded in 2018 by Benjamin Chee HH. Specializes in classical dress watches with vintage-inspired design, including the Merveilleux collection featuring 1950s teardrop lug cases and Art Deco sector dials. Offers both standard handcrafted watches and a Haute Horlogerie Division using platinum, rose gold, and Swiss haute horlogerie movements from Vaucher Manufacture Fleurier.</v>
       </c>
     </row>
     <row r="77">
@@ -36353,7 +36353,7 @@
         <v>Singapore</v>
       </c>
       <c r="C80" t="str">
-        <v/>
+        <v>Singapore</v>
       </c>
       <c r="D80" t="str">
         <v/>
@@ -36737,7 +36737,7 @@
         <v>Active</v>
       </c>
       <c r="H89" t="str">
-        <v/>
+        <v>Chronograph C-08</v>
       </c>
       <c r="I89" t="str">
         <v>2025-01-01</v>
@@ -36763,7 +36763,7 @@
         <v>Hong Kong</v>
       </c>
       <c r="C90" t="str">
-        <v/>
+        <v>Kowloon</v>
       </c>
       <c r="D90" t="str">
         <v/>
@@ -36806,14 +36806,14 @@
       <c r="C91" t="str">
         <v>Seoul</v>
       </c>
-      <c r="D91" t="str">
-        <v/>
+      <c r="D91">
+        <v>2021</v>
       </c>
       <c r="E91">
         <v>875</v>
       </c>
-      <c r="F91" t="str">
-        <v/>
+      <c r="F91">
+        <v>1499</v>
       </c>
       <c r="G91" t="str">
         <v>Active</v>
@@ -36828,7 +36828,7 @@
         <v>https://www.pitzmann.com/</v>
       </c>
       <c r="K91" t="str">
-        <v/>
+        <v>pitzmann_official</v>
       </c>
       <c r="L91" t="str">
         <v>MBWDB</v>
@@ -36968,7 +36968,7 @@
         <v>China</v>
       </c>
       <c r="C95" t="str">
-        <v/>
+        <v>Roma</v>
       </c>
       <c r="D95">
         <v>2019</v>
@@ -37088,10 +37088,10 @@
         <v>Relax</v>
       </c>
       <c r="B98" t="str">
-        <v>United States</v>
+        <v>China</v>
       </c>
       <c r="C98" t="str">
-        <v/>
+        <v>Guangzhou</v>
       </c>
       <c r="D98" t="str">
         <v/>
@@ -37132,7 +37132,7 @@
         <v>Singapore</v>
       </c>
       <c r="C99" t="str">
-        <v/>
+        <v>Singapore</v>
       </c>
       <c r="D99">
         <v>2014</v>
@@ -37173,7 +37173,7 @@
         <v>Hong Kong</v>
       </c>
       <c r="C100" t="str">
-        <v/>
+        <v>Hong Kong</v>
       </c>
       <c r="D100" t="str">
         <v/>
@@ -37244,7 +37244,7 @@
         <v>MBWDB</v>
       </c>
       <c r="M101" t="str">
-        <v>Unknown brand — manual review needed</v>
+        <v>Singapore-based watch brand founded in 2020, specializing in titanium sports watches inspired by aerospace engineering. Known for durable adventure timepieces with UltraHEX™ titanium construction and models like Resolute, Valour, and Urbanist.</v>
       </c>
     </row>
     <row r="102">
@@ -37342,26 +37342,26 @@
       <c r="D104" t="str">
         <v/>
       </c>
-      <c r="E104" t="str">
-        <v/>
-      </c>
-      <c r="F104" t="str">
-        <v/>
+      <c r="E104">
+        <v>189</v>
+      </c>
+      <c r="F104">
+        <v>499</v>
       </c>
       <c r="G104" t="str">
         <v>Active</v>
       </c>
       <c r="H104" t="str">
-        <v/>
+        <v>MoonPhase Chrono Master S468</v>
       </c>
       <c r="I104" t="str">
-        <v/>
+        <v>2024-01-01</v>
       </c>
       <c r="J104" t="str">
         <v>https://sugesswatch.com/</v>
       </c>
       <c r="K104" t="str">
-        <v/>
+        <v>sugess_watches</v>
       </c>
       <c r="L104" t="str">
         <v>MBWDB</v>
@@ -37542,7 +37542,7 @@
         <v>South Korea</v>
       </c>
       <c r="C109" t="str">
-        <v/>
+        <v>Seoul</v>
       </c>
       <c r="D109">
         <v>2017</v>
@@ -37588,26 +37588,26 @@
       <c r="D110" t="str">
         <v/>
       </c>
-      <c r="E110" t="str">
-        <v/>
-      </c>
-      <c r="F110" t="str">
-        <v/>
+      <c r="E110">
+        <v>208</v>
+      </c>
+      <c r="F110">
+        <v>640</v>
       </c>
       <c r="G110" t="str">
         <v>Active</v>
       </c>
       <c r="H110" t="str">
-        <v/>
+        <v>Fair Lady</v>
       </c>
       <c r="I110" t="str">
-        <v/>
+        <v>2024-10-01</v>
       </c>
       <c r="J110" t="str">
         <v>https://solvil-et-titus.sg/</v>
       </c>
       <c r="K110" t="str">
-        <v/>
+        <v>solvilettitussg</v>
       </c>
       <c r="L110" t="str">
         <v>MBWDB</v>
@@ -37747,7 +37747,7 @@
         <v>Singapore</v>
       </c>
       <c r="C114" t="str">
-        <v/>
+        <v>Singapore</v>
       </c>
       <c r="D114">
         <v>2014</v>
@@ -37834,11 +37834,11 @@
       <c r="D116">
         <v>2021</v>
       </c>
-      <c r="E116" t="str">
-        <v/>
-      </c>
-      <c r="F116" t="str">
-        <v/>
+      <c r="E116">
+        <v>66</v>
+      </c>
+      <c r="F116">
+        <v>3000</v>
       </c>
       <c r="G116" t="str">
         <v>Active</v>
@@ -37853,7 +37853,7 @@
         <v>https://wancherwatch.com/</v>
       </c>
       <c r="K116" t="str">
-        <v/>
+        <v>wancherwatch_official</v>
       </c>
       <c r="L116" t="str">
         <v>MBWDB</v>
@@ -39864,7 +39864,7 @@
         <v>Switzerland</v>
       </c>
       <c r="C39" t="str">
-        <v/>
+        <v>Bangkok</v>
       </c>
       <c r="D39" t="str">
         <v/>
@@ -40804,7 +40804,7 @@
         <v>Cronos</v>
       </c>
       <c r="B62" t="str">
-        <v/>
+        <v>China</v>
       </c>
       <c r="C62" t="str">
         <v/>
@@ -44638,7 +44638,7 @@
         <v>Invader</v>
       </c>
       <c r="I155" t="str">
-        <v/>
+        <v>2026-01-01</v>
       </c>
       <c r="J155" t="str">
         <v>https://poshmark.com/brand/MAGICO-Men</v>
@@ -45276,7 +45276,7 @@
         <v>Singapore</v>
       </c>
       <c r="C171" t="str">
-        <v/>
+        <v>Singapore</v>
       </c>
       <c r="D171">
         <v>2019</v>
@@ -50811,7 +50811,7 @@
         <v>United States</v>
       </c>
       <c r="C306" t="str">
-        <v>Los Angeles</v>
+        <v>Austin</v>
       </c>
       <c r="D306" t="str">
         <v/>
@@ -51386,7 +51386,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B76"/>
+  <dimension ref="A1:B74"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -51525,7 +51525,7 @@
         <v>Brazil</v>
       </c>
       <c r="B17">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -51541,7 +51541,7 @@
         <v>Canada</v>
       </c>
       <c r="B19">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20">
@@ -51557,7 +51557,7 @@
         <v>China</v>
       </c>
       <c r="B21">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22">
@@ -51573,7 +51573,7 @@
         <v>Czech Republic</v>
       </c>
       <c r="B23">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24">
@@ -51581,76 +51581,76 @@
         <v>Denmark</v>
       </c>
       <c r="B24">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>England</v>
+        <v>Finland</v>
       </c>
       <c r="B25">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Finland</v>
+        <v>France</v>
       </c>
       <c r="B26">
-        <v>2</v>
+        <v>76</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>France</v>
+        <v>France and Switzerland</v>
       </c>
       <c r="B27">
-        <v>80</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>France and Switzerland</v>
+        <v>Germany</v>
       </c>
       <c r="B28">
-        <v>1</v>
+        <v>86</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Germany</v>
+        <v>Hong Kong</v>
       </c>
       <c r="B29">
-        <v>87</v>
+        <v>26</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Hong Kong</v>
+        <v>Hungary</v>
       </c>
       <c r="B30">
-        <v>25</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Hungary</v>
+        <v>Iceland</v>
       </c>
       <c r="B31">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Iceland</v>
+        <v>India</v>
       </c>
       <c r="B32">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>India</v>
+        <v>Indonesia</v>
       </c>
       <c r="B33">
         <v>5</v>
@@ -51658,119 +51658,119 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Indonesia</v>
+        <v>Ireland</v>
       </c>
       <c r="B34">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Ireland</v>
+        <v>Israel</v>
       </c>
       <c r="B35">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Israel</v>
+        <v>Italy</v>
       </c>
       <c r="B36">
-        <v>1</v>
+        <v>46</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Italy</v>
+        <v>Jamaica</v>
       </c>
       <c r="B37">
-        <v>48</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Jamaica</v>
+        <v>Japan</v>
       </c>
       <c r="B38">
-        <v>1</v>
+        <v>22</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Japan</v>
+        <v>Jordan</v>
       </c>
       <c r="B39">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Jordan</v>
+        <v>Lithuania</v>
       </c>
       <c r="B40">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Lithuania</v>
+        <v>Macau</v>
       </c>
       <c r="B41">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Macau</v>
+        <v>Malaysia</v>
       </c>
       <c r="B42">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Malaysia</v>
+        <v>Netherlands</v>
       </c>
       <c r="B43">
-        <v>6</v>
+        <v>25</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Netherlands</v>
+        <v>New Zealand</v>
       </c>
       <c r="B44">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>New Zealand</v>
+        <v>Norway</v>
       </c>
       <c r="B45">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Norway</v>
+        <v>null</v>
       </c>
       <c r="B46">
-        <v>9</v>
+        <v>138</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>null</v>
+        <v>Pakistan</v>
       </c>
       <c r="B47">
-        <v>139</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Pakistan</v>
+        <v>Peru</v>
       </c>
       <c r="B48">
         <v>1</v>
@@ -51778,39 +51778,39 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Peru</v>
+        <v>Philippines</v>
       </c>
       <c r="B49">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Philippines</v>
+        <v>Poland</v>
       </c>
       <c r="B50">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Poland</v>
+        <v>Portugal</v>
       </c>
       <c r="B51">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Portugal</v>
+        <v>Puerto Rico</v>
       </c>
       <c r="B52">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Puerto Rico</v>
+        <v>Romania</v>
       </c>
       <c r="B53">
         <v>2</v>
@@ -51818,31 +51818,31 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Romania</v>
+        <v>Russia</v>
       </c>
       <c r="B54">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Russia</v>
+        <v>Singapore</v>
       </c>
       <c r="B55">
-        <v>11</v>
+        <v>29</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Singapore</v>
+        <v>Slovakia</v>
       </c>
       <c r="B56">
-        <v>29</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Slovakia</v>
+        <v>Slovenia</v>
       </c>
       <c r="B57">
         <v>1</v>
@@ -51850,95 +51850,95 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Slovenia</v>
+        <v>South Africa</v>
       </c>
       <c r="B58">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>South Africa</v>
+        <v>South Korea</v>
       </c>
       <c r="B59">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>South Korea</v>
+        <v>Soviet Union</v>
       </c>
       <c r="B60">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Soviet Union</v>
+        <v>Spain</v>
       </c>
       <c r="B61">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Spain</v>
+        <v>Sweden</v>
       </c>
       <c r="B62">
-        <v>6</v>
+        <v>19</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Sweden</v>
+        <v>Switzerland</v>
       </c>
       <c r="B63">
-        <v>21</v>
+        <v>177</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Switzerland</v>
+        <v>Taiwan</v>
       </c>
       <c r="B64">
-        <v>177</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Taiwan</v>
+        <v>Thailand</v>
       </c>
       <c r="B65">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Thailand</v>
+        <v>United Kingdom</v>
       </c>
       <c r="B66">
-        <v>4</v>
+        <v>110</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>United Kingdom</v>
+        <v>United States</v>
       </c>
       <c r="B67">
-        <v>108</v>
+        <v>224</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>United States</v>
+        <v>Unknown</v>
       </c>
       <c r="B68">
-        <v>222</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Unknown</v>
+        <v>Vietnam</v>
       </c>
       <c r="B69">
         <v>1</v>
@@ -51946,63 +51946,47 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>USA</v>
-      </c>
-      <c r="B70">
-        <v>2</v>
+        <v/>
+      </c>
+      <c r="B70" t="str">
+        <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Vietnam</v>
-      </c>
-      <c r="B71">
-        <v>1</v>
+        <v>Status</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Count</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v/>
-      </c>
-      <c r="B72" t="str">
-        <v/>
+        <v>Active</v>
+      </c>
+      <c r="B72">
+        <v>1236</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Status</v>
-      </c>
-      <c r="B73" t="str">
-        <v>Count</v>
+        <v>Dormant</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Active</v>
+        <v>Defunct</v>
       </c>
       <c r="B74">
-        <v>1236</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="str">
-        <v>Dormant</v>
-      </c>
-      <c r="B75">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="str">
-        <v>Defunct</v>
-      </c>
-      <c r="B76">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B76"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B74"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>